<commit_message>
docs(correcciones): estado de la fase 1 en el Excel del reparto
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Correcciones/Reparto_Correcciones.xlsx
+++ b/Correcciones/Reparto_Correcciones.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/04056fffbf4849c6/Desktop/Estudios/Ingenieria en Sistemas/Ultimo Cuatri/Implantacion/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8F8D4389-595E-4CF9-BD61-29F667513908}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="48" documentId="8_{8F8D4389-595E-4CF9-BD61-29F667513908}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{479AA629-332A-4350-BE21-47EF3B914DB9}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{02318C6D-03B9-4FBB-AC05-EEF1D4A56137}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{02318C6D-03B9-4FBB-AC05-EEF1D4A56137}"/>
   </bookViews>
   <sheets>
     <sheet name="Resumen" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Paquete 3 - Gerald'!$A$4:$I$18</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Paquete 4 - David'!$A$4:$I$21</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="757" uniqueCount="384">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="781" uniqueCount="409">
   <si>
     <t>Reparto de correcciones — Distribuidora JJ / Licorera La Bodega</t>
   </si>
@@ -1218,6 +1218,81 @@
   </si>
   <si>
     <t>al presionar "Exportar" sobre los resultados el sistema descarga los resultados en formato Excel (.xlsx).</t>
+  </si>
+  <si>
+    <t>Corregido</t>
+  </si>
+  <si>
+    <t>Procedimientos de productos con el contrato de la app. Migración 0210</t>
+  </si>
+  <si>
+    <t>Fecha de vencimiento y advertencia a 30 días. Migración 0211</t>
+  </si>
+  <si>
+    <t>No se inactiva un producto con stock</t>
+  </si>
+  <si>
+    <t>Búsqueda por SKU. Migración 0212</t>
+  </si>
+  <si>
+    <t>Verificación diaria automática (servicio en segundo plano)</t>
+  </si>
+  <si>
+    <t>Rechaza promociones traslapadas. Migración 0213</t>
+  </si>
+  <si>
+    <t>Límite de unidades con inactivación automática. El pedido que cruza el límite conserva el descuento. Migración 0214</t>
+  </si>
+  <si>
+    <t>Mensajes de validación visibles al crear combo</t>
+  </si>
+  <si>
+    <t>Misma causa que BUG-09-03 (0200)</t>
+  </si>
+  <si>
+    <t>sp_Admin_GetOrderHeader restaurado al contrato correcto. Migración 0200</t>
+  </si>
+  <si>
+    <t>Egresos leídos de GastosOperativos (la tabla Gastos no existe)</t>
+  </si>
+  <si>
+    <t>Misma causa que BUG-09-03 + Venta móvil envía el comprobante</t>
+  </si>
+  <si>
+    <t>Comprobante por WhatsApp (enlace wa.me, un clic) al facturar y en el detalle. Migración 0201</t>
+  </si>
+  <si>
+    <t>La API informa el resultado real. En Azure faltan las variables SMTP (al cierre)</t>
+  </si>
+  <si>
+    <t>Confirmación al cliente y aviso de resolución por correo</t>
+  </si>
+  <si>
+    <t>Indica que el correo no está registrado, como pide la HU</t>
+  </si>
+  <si>
+    <t>Mensaje controlado de espera en lugar de 429</t>
+  </si>
+  <si>
+    <t>Token antifalsificación en la cabecera correcta</t>
+  </si>
+  <si>
+    <t>La app guarda clientes y productos para vender sin conexión</t>
+  </si>
+  <si>
+    <t>La app actualiza el pedido a EnRuta/Fallido. Migración 0220. Gerald debe llamar al mismo SP desde la web</t>
+  </si>
+  <si>
+    <t>Mapa interactivo con la secuencia de visitas</t>
+  </si>
+  <si>
+    <t>Aviso al chofer al asignar la ruta. Migración 0221</t>
+  </si>
+  <si>
+    <t>Parcial: Aviso en el celular al abrir o volver a la app; con la app cerrada requiere Firebase. Migración 0222</t>
+  </si>
+  <si>
+    <t>Aviso al chofer al reasignar la ruta (campana web y app). Migración 0221</t>
   </si>
 </sst>
 </file>
@@ -1400,9 +1475,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
@@ -1411,9 +1483,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -1428,10 +1497,6 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1441,9 +1506,6 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -1506,6 +1568,19 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1930,7 +2005,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:I36"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="14.7109375" customWidth="1"/>
     <col min="3" max="3" width="40.7109375" customWidth="1"/>
@@ -1945,518 +2020,518 @@
       </c>
     </row>
     <row r="2" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="20" t="s">
+      <c r="A2" s="39" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="20"/>
-      <c r="C2" s="20"/>
-      <c r="D2" s="20"/>
-      <c r="E2" s="20"/>
-      <c r="F2" s="20"/>
-      <c r="G2" s="20"/>
-      <c r="H2" s="20"/>
-      <c r="I2" s="20"/>
+      <c r="B2" s="39"/>
+      <c r="C2" s="39"/>
+      <c r="D2" s="39"/>
+      <c r="E2" s="39"/>
+      <c r="F2" s="39"/>
+      <c r="G2" s="39"/>
+      <c r="H2" s="39"/>
+      <c r="I2" s="39"/>
     </row>
     <row r="4" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="F4" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="G4" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="H4" s="3" t="s">
+      <c r="H4" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="I4" s="3" t="s">
+      <c r="I4" s="11" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="156" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="D5" s="9">
+      <c r="D5" s="7">
         <v>44</v>
       </c>
-      <c r="E5" s="9">
+      <c r="E5" s="7">
         <v>6</v>
       </c>
-      <c r="F5" s="9">
+      <c r="F5" s="7">
         <v>7</v>
       </c>
-      <c r="G5" s="9">
+      <c r="G5" s="7">
         <v>31</v>
       </c>
-      <c r="H5" s="9">
+      <c r="H5" s="7">
         <v>96</v>
       </c>
-      <c r="I5" s="5" t="s">
+      <c r="I5" s="4" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="51" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="6" t="s">
+      <c r="A6" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="D6" s="10">
+      <c r="D6" s="8">
         <v>16</v>
       </c>
-      <c r="E6" s="10">
+      <c r="E6" s="8">
         <v>1</v>
       </c>
-      <c r="F6" s="10">
+      <c r="F6" s="8">
         <v>8</v>
       </c>
-      <c r="G6" s="10">
+      <c r="G6" s="8">
         <v>7</v>
       </c>
-      <c r="H6" s="10">
+      <c r="H6" s="8">
         <v>36</v>
       </c>
-      <c r="I6" s="7" t="s">
+      <c r="I6" s="12" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="66" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="6" t="s">
+      <c r="A7" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C7" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="D7" s="10">
+      <c r="D7" s="8">
         <v>14</v>
       </c>
-      <c r="E7" s="10">
+      <c r="E7" s="8">
         <v>0</v>
       </c>
-      <c r="F7" s="10">
+      <c r="F7" s="8">
         <v>3</v>
       </c>
-      <c r="G7" s="10">
+      <c r="G7" s="8">
         <v>11</v>
       </c>
-      <c r="H7" s="10">
+      <c r="H7" s="8">
         <v>25</v>
       </c>
-      <c r="I7" s="7" t="s">
+      <c r="I7" s="12" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="66" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="6" t="s">
+      <c r="A8" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="B8" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="C8" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="D8" s="10">
+      <c r="D8" s="8">
         <v>17</v>
       </c>
-      <c r="E8" s="10">
+      <c r="E8" s="8">
         <v>0</v>
       </c>
-      <c r="F8" s="10">
+      <c r="F8" s="8">
         <v>1</v>
       </c>
-      <c r="G8" s="10">
+      <c r="G8" s="8">
         <v>16</v>
       </c>
-      <c r="H8" s="10">
+      <c r="H8" s="8">
         <v>26</v>
       </c>
-      <c r="I8" s="7" t="s">
+      <c r="I8" s="12" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A9" s="8" t="s">
+      <c r="A9" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="B9" s="8"/>
-      <c r="C9" s="8"/>
-      <c r="D9" s="11">
+      <c r="B9" s="6"/>
+      <c r="C9" s="6"/>
+      <c r="D9" s="9">
         <f>SUM(D5:D8)</f>
         <v>91</v>
       </c>
-      <c r="E9" s="11">
+      <c r="E9" s="9">
         <f>SUM(E5:E8)</f>
         <v>7</v>
       </c>
-      <c r="F9" s="11">
+      <c r="F9" s="9">
         <f>SUM(F5:F8)</f>
         <v>19</v>
       </c>
-      <c r="G9" s="11">
+      <c r="G9" s="9">
         <f>SUM(G5:G8)</f>
         <v>65</v>
       </c>
-      <c r="H9" s="11">
+      <c r="H9" s="9">
         <f>SUM(H5:H8)</f>
         <v>183</v>
       </c>
-      <c r="I9" s="8"/>
+      <c r="I9" s="6"/>
     </row>
     <row r="11" spans="1:9" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A11" s="12" t="s">
+      <c r="A11" s="10" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="14" t="s">
+      <c r="A12" s="37" t="s">
         <v>29</v>
       </c>
-      <c r="B12" s="14"/>
-      <c r="C12" s="14"/>
-      <c r="D12" s="14"/>
-      <c r="E12" s="14"/>
-      <c r="F12" s="14"/>
-      <c r="G12" s="14"/>
-      <c r="H12" s="14"/>
-      <c r="I12" s="14"/>
+      <c r="B12" s="37"/>
+      <c r="C12" s="37"/>
+      <c r="D12" s="37"/>
+      <c r="E12" s="37"/>
+      <c r="F12" s="37"/>
+      <c r="G12" s="37"/>
+      <c r="H12" s="37"/>
+      <c r="I12" s="37"/>
     </row>
     <row r="13" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="14" t="s">
+      <c r="A13" s="37" t="s">
         <v>30</v>
       </c>
-      <c r="B13" s="14"/>
-      <c r="C13" s="14"/>
-      <c r="D13" s="14"/>
-      <c r="E13" s="14"/>
-      <c r="F13" s="14"/>
-      <c r="G13" s="14"/>
-      <c r="H13" s="14"/>
-      <c r="I13" s="14"/>
+      <c r="B13" s="37"/>
+      <c r="C13" s="37"/>
+      <c r="D13" s="37"/>
+      <c r="E13" s="37"/>
+      <c r="F13" s="37"/>
+      <c r="G13" s="37"/>
+      <c r="H13" s="37"/>
+      <c r="I13" s="37"/>
     </row>
     <row r="14" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="14" t="s">
+      <c r="A14" s="37" t="s">
         <v>31</v>
       </c>
-      <c r="B14" s="14"/>
-      <c r="C14" s="14"/>
-      <c r="D14" s="14"/>
-      <c r="E14" s="14"/>
-      <c r="F14" s="14"/>
-      <c r="G14" s="14"/>
-      <c r="H14" s="14"/>
-      <c r="I14" s="14"/>
+      <c r="B14" s="37"/>
+      <c r="C14" s="37"/>
+      <c r="D14" s="37"/>
+      <c r="E14" s="37"/>
+      <c r="F14" s="37"/>
+      <c r="G14" s="37"/>
+      <c r="H14" s="37"/>
+      <c r="I14" s="37"/>
     </row>
     <row r="15" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="14" t="s">
+      <c r="A15" s="37" t="s">
         <v>32</v>
       </c>
-      <c r="B15" s="14"/>
-      <c r="C15" s="14"/>
-      <c r="D15" s="14"/>
-      <c r="E15" s="14"/>
-      <c r="F15" s="14"/>
-      <c r="G15" s="14"/>
-      <c r="H15" s="14"/>
-      <c r="I15" s="14"/>
+      <c r="B15" s="37"/>
+      <c r="C15" s="37"/>
+      <c r="D15" s="37"/>
+      <c r="E15" s="37"/>
+      <c r="F15" s="37"/>
+      <c r="G15" s="37"/>
+      <c r="H15" s="37"/>
+      <c r="I15" s="37"/>
     </row>
     <row r="16" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="14" t="s">
+      <c r="A16" s="37" t="s">
         <v>33</v>
       </c>
-      <c r="B16" s="14"/>
-      <c r="C16" s="14"/>
-      <c r="D16" s="14"/>
-      <c r="E16" s="14"/>
-      <c r="F16" s="14"/>
-      <c r="G16" s="14"/>
-      <c r="H16" s="14"/>
-      <c r="I16" s="14"/>
+      <c r="B16" s="37"/>
+      <c r="C16" s="37"/>
+      <c r="D16" s="37"/>
+      <c r="E16" s="37"/>
+      <c r="F16" s="37"/>
+      <c r="G16" s="37"/>
+      <c r="H16" s="37"/>
+      <c r="I16" s="37"/>
     </row>
     <row r="17" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="14" t="s">
+      <c r="A17" s="37" t="s">
         <v>34</v>
       </c>
-      <c r="B17" s="14"/>
-      <c r="C17" s="14"/>
-      <c r="D17" s="14"/>
-      <c r="E17" s="14"/>
-      <c r="F17" s="14"/>
-      <c r="G17" s="14"/>
-      <c r="H17" s="14"/>
-      <c r="I17" s="14"/>
+      <c r="B17" s="37"/>
+      <c r="C17" s="37"/>
+      <c r="D17" s="37"/>
+      <c r="E17" s="37"/>
+      <c r="F17" s="37"/>
+      <c r="G17" s="37"/>
+      <c r="H17" s="37"/>
+      <c r="I17" s="37"/>
     </row>
     <row r="18" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="14" t="s">
+      <c r="A18" s="37" t="s">
         <v>35</v>
       </c>
-      <c r="B18" s="14"/>
-      <c r="C18" s="14"/>
-      <c r="D18" s="14"/>
-      <c r="E18" s="14"/>
-      <c r="F18" s="14"/>
-      <c r="G18" s="14"/>
-      <c r="H18" s="14"/>
-      <c r="I18" s="14"/>
+      <c r="B18" s="37"/>
+      <c r="C18" s="37"/>
+      <c r="D18" s="37"/>
+      <c r="E18" s="37"/>
+      <c r="F18" s="37"/>
+      <c r="G18" s="37"/>
+      <c r="H18" s="37"/>
+      <c r="I18" s="37"/>
     </row>
     <row r="20" spans="1:9" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A20" s="12" t="s">
+      <c r="A20" s="10" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A21" s="3" t="s">
+      <c r="A21" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="B21" s="3" t="s">
+      <c r="B21" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="C21" s="15" t="s">
+      <c r="C21" s="41" t="s">
         <v>39</v>
       </c>
-      <c r="D21" s="15"/>
-      <c r="E21" s="15"/>
-      <c r="F21" s="15"/>
-      <c r="G21" s="15"/>
-      <c r="H21" s="15"/>
-      <c r="I21" s="15"/>
+      <c r="D21" s="41"/>
+      <c r="E21" s="41"/>
+      <c r="F21" s="41"/>
+      <c r="G21" s="41"/>
+      <c r="H21" s="41"/>
+      <c r="I21" s="41"/>
     </row>
     <row r="22" spans="1:9" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="6" t="s">
+      <c r="A22" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="B22" s="6" t="s">
+      <c r="B22" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="C22" s="16" t="s">
+      <c r="C22" s="40" t="s">
         <v>42</v>
       </c>
-      <c r="D22" s="16"/>
-      <c r="E22" s="16"/>
-      <c r="F22" s="16"/>
-      <c r="G22" s="16"/>
-      <c r="H22" s="16"/>
-      <c r="I22" s="16"/>
+      <c r="D22" s="40"/>
+      <c r="E22" s="40"/>
+      <c r="F22" s="40"/>
+      <c r="G22" s="40"/>
+      <c r="H22" s="40"/>
+      <c r="I22" s="40"/>
     </row>
     <row r="23" spans="1:9" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="6" t="s">
+      <c r="A23" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="B23" s="6" t="s">
+      <c r="B23" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="C23" s="16" t="s">
+      <c r="C23" s="40" t="s">
         <v>44</v>
       </c>
-      <c r="D23" s="16"/>
-      <c r="E23" s="16"/>
-      <c r="F23" s="16"/>
-      <c r="G23" s="16"/>
-      <c r="H23" s="16"/>
-      <c r="I23" s="16"/>
+      <c r="D23" s="40"/>
+      <c r="E23" s="40"/>
+      <c r="F23" s="40"/>
+      <c r="G23" s="40"/>
+      <c r="H23" s="40"/>
+      <c r="I23" s="40"/>
     </row>
     <row r="24" spans="1:9" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="6" t="s">
+      <c r="A24" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="B24" s="6" t="s">
+      <c r="B24" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="C24" s="16" t="s">
+      <c r="C24" s="40" t="s">
         <v>47</v>
       </c>
-      <c r="D24" s="16"/>
-      <c r="E24" s="16"/>
-      <c r="F24" s="16"/>
-      <c r="G24" s="16"/>
-      <c r="H24" s="16"/>
-      <c r="I24" s="16"/>
+      <c r="D24" s="40"/>
+      <c r="E24" s="40"/>
+      <c r="F24" s="40"/>
+      <c r="G24" s="40"/>
+      <c r="H24" s="40"/>
+      <c r="I24" s="40"/>
     </row>
     <row r="25" spans="1:9" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="6" t="s">
+      <c r="A25" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="B25" s="6" t="s">
+      <c r="B25" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="C25" s="16" t="s">
+      <c r="C25" s="40" t="s">
         <v>49</v>
       </c>
-      <c r="D25" s="16"/>
-      <c r="E25" s="16"/>
-      <c r="F25" s="16"/>
-      <c r="G25" s="16"/>
-      <c r="H25" s="16"/>
-      <c r="I25" s="16"/>
+      <c r="D25" s="40"/>
+      <c r="E25" s="40"/>
+      <c r="F25" s="40"/>
+      <c r="G25" s="40"/>
+      <c r="H25" s="40"/>
+      <c r="I25" s="40"/>
     </row>
     <row r="26" spans="1:9" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="6" t="s">
+      <c r="A26" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="B26" s="6" t="s">
+      <c r="B26" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="C26" s="16" t="s">
+      <c r="C26" s="40" t="s">
         <v>52</v>
       </c>
-      <c r="D26" s="16"/>
-      <c r="E26" s="16"/>
-      <c r="F26" s="16"/>
-      <c r="G26" s="16"/>
-      <c r="H26" s="16"/>
-      <c r="I26" s="16"/>
+      <c r="D26" s="40"/>
+      <c r="E26" s="40"/>
+      <c r="F26" s="40"/>
+      <c r="G26" s="40"/>
+      <c r="H26" s="40"/>
+      <c r="I26" s="40"/>
     </row>
     <row r="28" spans="1:9" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A28" s="12" t="s">
+      <c r="A28" s="10" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A29" s="17" t="s">
+      <c r="A29" s="13" t="s">
         <v>54</v>
       </c>
-      <c r="B29" s="13" t="s">
+      <c r="B29" s="38" t="s">
         <v>55</v>
       </c>
-      <c r="C29" s="13"/>
-      <c r="D29" s="13"/>
-      <c r="E29" s="13"/>
-      <c r="F29" s="13"/>
-      <c r="G29" s="13"/>
-      <c r="H29" s="13"/>
-      <c r="I29" s="13"/>
+      <c r="C29" s="38"/>
+      <c r="D29" s="38"/>
+      <c r="E29" s="38"/>
+      <c r="F29" s="38"/>
+      <c r="G29" s="38"/>
+      <c r="H29" s="38"/>
+      <c r="I29" s="38"/>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A30" s="18" t="s">
+      <c r="A30" s="14" t="s">
         <v>56</v>
       </c>
-      <c r="B30" s="13" t="s">
+      <c r="B30" s="38" t="s">
         <v>57</v>
       </c>
-      <c r="C30" s="13"/>
-      <c r="D30" s="13"/>
-      <c r="E30" s="13"/>
-      <c r="F30" s="13"/>
-      <c r="G30" s="13"/>
-      <c r="H30" s="13"/>
-      <c r="I30" s="13"/>
+      <c r="C30" s="38"/>
+      <c r="D30" s="38"/>
+      <c r="E30" s="38"/>
+      <c r="F30" s="38"/>
+      <c r="G30" s="38"/>
+      <c r="H30" s="38"/>
+      <c r="I30" s="38"/>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A31" s="19" t="s">
+      <c r="A31" s="15" t="s">
         <v>58</v>
       </c>
-      <c r="B31" s="13" t="s">
+      <c r="B31" s="38" t="s">
         <v>59</v>
       </c>
-      <c r="C31" s="13"/>
-      <c r="D31" s="13"/>
-      <c r="E31" s="13"/>
-      <c r="F31" s="13"/>
-      <c r="G31" s="13"/>
-      <c r="H31" s="13"/>
-      <c r="I31" s="13"/>
+      <c r="C31" s="38"/>
+      <c r="D31" s="38"/>
+      <c r="E31" s="38"/>
+      <c r="F31" s="38"/>
+      <c r="G31" s="38"/>
+      <c r="H31" s="38"/>
+      <c r="I31" s="38"/>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="B32" s="13" t="s">
+      <c r="B32" s="38" t="s">
         <v>61</v>
       </c>
-      <c r="C32" s="13"/>
-      <c r="D32" s="13"/>
-      <c r="E32" s="13"/>
-      <c r="F32" s="13"/>
-      <c r="G32" s="13"/>
-      <c r="H32" s="13"/>
-      <c r="I32" s="13"/>
+      <c r="C32" s="38"/>
+      <c r="D32" s="38"/>
+      <c r="E32" s="38"/>
+      <c r="F32" s="38"/>
+      <c r="G32" s="38"/>
+      <c r="H32" s="38"/>
+      <c r="I32" s="38"/>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="B33" s="13" t="s">
+      <c r="B33" s="38" t="s">
         <v>63</v>
       </c>
-      <c r="C33" s="13"/>
-      <c r="D33" s="13"/>
-      <c r="E33" s="13"/>
-      <c r="F33" s="13"/>
-      <c r="G33" s="13"/>
-      <c r="H33" s="13"/>
-      <c r="I33" s="13"/>
+      <c r="C33" s="38"/>
+      <c r="D33" s="38"/>
+      <c r="E33" s="38"/>
+      <c r="F33" s="38"/>
+      <c r="G33" s="38"/>
+      <c r="H33" s="38"/>
+      <c r="I33" s="38"/>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="B34" s="13" t="s">
+      <c r="B34" s="38" t="s">
         <v>65</v>
       </c>
-      <c r="C34" s="13"/>
-      <c r="D34" s="13"/>
-      <c r="E34" s="13"/>
-      <c r="F34" s="13"/>
-      <c r="G34" s="13"/>
-      <c r="H34" s="13"/>
-      <c r="I34" s="13"/>
+      <c r="C34" s="38"/>
+      <c r="D34" s="38"/>
+      <c r="E34" s="38"/>
+      <c r="F34" s="38"/>
+      <c r="G34" s="38"/>
+      <c r="H34" s="38"/>
+      <c r="I34" s="38"/>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B35" s="13" t="s">
+      <c r="B35" s="38" t="s">
         <v>66</v>
       </c>
-      <c r="C35" s="13"/>
-      <c r="D35" s="13"/>
-      <c r="E35" s="13"/>
-      <c r="F35" s="13"/>
-      <c r="G35" s="13"/>
-      <c r="H35" s="13"/>
-      <c r="I35" s="13"/>
+      <c r="C35" s="38"/>
+      <c r="D35" s="38"/>
+      <c r="E35" s="38"/>
+      <c r="F35" s="38"/>
+      <c r="G35" s="38"/>
+      <c r="H35" s="38"/>
+      <c r="I35" s="38"/>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="B36" s="13" t="s">
+      <c r="B36" s="38" t="s">
         <v>68</v>
       </c>
-      <c r="C36" s="13"/>
-      <c r="D36" s="13"/>
-      <c r="E36" s="13"/>
-      <c r="F36" s="13"/>
-      <c r="G36" s="13"/>
-      <c r="H36" s="13"/>
-      <c r="I36" s="13"/>
+      <c r="C36" s="38"/>
+      <c r="D36" s="38"/>
+      <c r="E36" s="38"/>
+      <c r="F36" s="38"/>
+      <c r="G36" s="38"/>
+      <c r="H36" s="38"/>
+      <c r="I36" s="38"/>
     </row>
   </sheetData>
   <mergeCells count="22">
@@ -2476,12 +2551,12 @@
     <mergeCell ref="C23:I23"/>
     <mergeCell ref="C24:I24"/>
     <mergeCell ref="C25:I25"/>
+    <mergeCell ref="A17:I17"/>
     <mergeCell ref="A12:I12"/>
     <mergeCell ref="A13:I13"/>
     <mergeCell ref="A14:I14"/>
     <mergeCell ref="A15:I15"/>
     <mergeCell ref="A16:I16"/>
-    <mergeCell ref="A17:I17"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup fitToHeight="0" orientation="landscape" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
@@ -2494,7 +2569,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:I50"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.7109375" customWidth="1"/>
     <col min="2" max="2" width="24.7109375" customWidth="1"/>
@@ -2512,1234 +2587,1282 @@
       </c>
     </row>
     <row r="2" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="20" t="s">
+      <c r="A2" s="39" t="s">
         <v>70</v>
       </c>
-      <c r="B2" s="20"/>
-      <c r="C2" s="20"/>
-      <c r="D2" s="20"/>
-      <c r="E2" s="20"/>
-      <c r="F2" s="20"/>
-      <c r="G2" s="20"/>
-      <c r="H2" s="20"/>
-      <c r="I2" s="20"/>
+      <c r="B2" s="39"/>
+      <c r="C2" s="39"/>
+      <c r="D2" s="39"/>
+      <c r="E2" s="39"/>
+      <c r="F2" s="39"/>
+      <c r="G2" s="39"/>
+      <c r="H2" s="39"/>
+      <c r="I2" s="39"/>
     </row>
     <row r="4" spans="1:9" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="11" t="s">
         <v>71</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="11" t="s">
         <v>73</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="11" t="s">
         <v>74</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="11" t="s">
         <v>75</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="F4" s="11" t="s">
         <v>76</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="G4" s="11" t="s">
         <v>77</v>
       </c>
-      <c r="H4" s="3" t="s">
+      <c r="H4" s="11" t="s">
         <v>78</v>
       </c>
-      <c r="I4" s="3" t="s">
+      <c r="I4" s="11" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="51" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="25">
+      <c r="A5" s="20">
         <v>1</v>
       </c>
-      <c r="B5" s="7" t="s">
+      <c r="B5" s="12" t="s">
         <v>80</v>
       </c>
-      <c r="C5" s="25" t="s">
+      <c r="C5" s="20" t="s">
         <v>81</v>
       </c>
-      <c r="D5" s="7" t="s">
+      <c r="D5" s="12" t="s">
         <v>82</v>
       </c>
-      <c r="E5" s="7" t="s">
+      <c r="E5" s="12" t="s">
         <v>83</v>
       </c>
-      <c r="F5" s="30" t="s">
+      <c r="F5" s="25" t="s">
         <v>84</v>
       </c>
-      <c r="G5" s="25" t="s">
+      <c r="G5" s="20" t="s">
         <v>85</v>
       </c>
-      <c r="H5" s="25" t="s">
-        <v>86</v>
-      </c>
-      <c r="I5" s="7"/>
+      <c r="H5" s="20" t="s">
+        <v>384</v>
+      </c>
+      <c r="I5" s="12" t="s">
+        <v>385</v>
+      </c>
     </row>
     <row r="6" spans="1:9" ht="66" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="25">
+      <c r="A6" s="20">
         <v>2</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="B6" s="12" t="s">
         <v>80</v>
       </c>
-      <c r="C6" s="25" t="s">
+      <c r="C6" s="20" t="s">
         <v>87</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="D6" s="12" t="s">
         <v>88</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="E6" s="12" t="s">
         <v>89</v>
       </c>
-      <c r="F6" s="31" t="s">
-        <v>90</v>
-      </c>
-      <c r="G6" s="25" t="s">
+      <c r="F6" s="26" t="s">
+        <v>90</v>
+      </c>
+      <c r="G6" s="20" t="s">
         <v>85</v>
       </c>
-      <c r="H6" s="25" t="s">
-        <v>86</v>
-      </c>
-      <c r="I6" s="7"/>
+      <c r="H6" s="20" t="s">
+        <v>384</v>
+      </c>
+      <c r="I6" s="12" t="s">
+        <v>386</v>
+      </c>
     </row>
     <row r="7" spans="1:9" ht="51" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="25">
+      <c r="A7" s="20">
         <v>3</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B7" s="12" t="s">
         <v>80</v>
       </c>
-      <c r="C7" s="25" t="s">
+      <c r="C7" s="20" t="s">
         <v>91</v>
       </c>
-      <c r="D7" s="7" t="s">
+      <c r="D7" s="12" t="s">
         <v>92</v>
       </c>
-      <c r="E7" s="7" t="s">
+      <c r="E7" s="12" t="s">
         <v>93</v>
       </c>
-      <c r="F7" s="31" t="s">
-        <v>90</v>
-      </c>
-      <c r="G7" s="25" t="s">
-        <v>90</v>
-      </c>
-      <c r="H7" s="25" t="s">
-        <v>86</v>
-      </c>
-      <c r="I7" s="7"/>
+      <c r="F7" s="26" t="s">
+        <v>90</v>
+      </c>
+      <c r="G7" s="20" t="s">
+        <v>90</v>
+      </c>
+      <c r="H7" s="20" t="s">
+        <v>384</v>
+      </c>
+      <c r="I7" s="12" t="s">
+        <v>387</v>
+      </c>
     </row>
     <row r="8" spans="1:9" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="25">
+      <c r="A8" s="20">
         <v>4</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="12" t="s">
         <v>80</v>
       </c>
-      <c r="C8" s="25" t="s">
+      <c r="C8" s="20" t="s">
         <v>94</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="D8" s="12" t="s">
         <v>95</v>
       </c>
-      <c r="E8" s="7" t="s">
+      <c r="E8" s="12" t="s">
         <v>96</v>
       </c>
-      <c r="F8" s="31" t="s">
-        <v>90</v>
-      </c>
-      <c r="G8" s="25" t="s">
+      <c r="F8" s="26" t="s">
+        <v>90</v>
+      </c>
+      <c r="G8" s="20" t="s">
         <v>97</v>
       </c>
-      <c r="H8" s="25" t="s">
-        <v>86</v>
-      </c>
-      <c r="I8" s="7"/>
+      <c r="H8" s="20" t="s">
+        <v>384</v>
+      </c>
+      <c r="I8" s="12" t="s">
+        <v>388</v>
+      </c>
     </row>
     <row r="9" spans="1:9" ht="66" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="26">
+      <c r="A9" s="21">
         <v>5</v>
       </c>
-      <c r="B9" s="23" t="s">
+      <c r="B9" s="18" t="s">
         <v>80</v>
       </c>
-      <c r="C9" s="26" t="s">
+      <c r="C9" s="21" t="s">
         <v>98</v>
       </c>
-      <c r="D9" s="23" t="s">
+      <c r="D9" s="18" t="s">
         <v>99</v>
       </c>
-      <c r="E9" s="23" t="s">
+      <c r="E9" s="18" t="s">
         <v>100</v>
       </c>
-      <c r="F9" s="32" t="s">
-        <v>90</v>
-      </c>
-      <c r="G9" s="26" t="s">
-        <v>90</v>
-      </c>
-      <c r="H9" s="26" t="s">
-        <v>86</v>
-      </c>
-      <c r="I9" s="23"/>
+      <c r="F9" s="27" t="s">
+        <v>90</v>
+      </c>
+      <c r="G9" s="21" t="s">
+        <v>90</v>
+      </c>
+      <c r="H9" s="21" t="s">
+        <v>384</v>
+      </c>
+      <c r="I9" s="18" t="s">
+        <v>389</v>
+      </c>
     </row>
     <row r="10" spans="1:9" ht="51" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="27">
+      <c r="A10" s="22">
         <v>6</v>
       </c>
-      <c r="B10" s="24" t="s">
+      <c r="B10" s="19" t="s">
         <v>101</v>
       </c>
-      <c r="C10" s="27" t="s">
+      <c r="C10" s="22" t="s">
         <v>102</v>
       </c>
-      <c r="D10" s="24" t="s">
+      <c r="D10" s="19" t="s">
         <v>103</v>
       </c>
-      <c r="E10" s="24" t="s">
+      <c r="E10" s="19" t="s">
         <v>104</v>
       </c>
-      <c r="F10" s="33" t="s">
+      <c r="F10" s="28" t="s">
         <v>85</v>
       </c>
-      <c r="G10" s="27" t="s">
-        <v>90</v>
-      </c>
-      <c r="H10" s="27" t="s">
-        <v>86</v>
-      </c>
-      <c r="I10" s="24"/>
+      <c r="G10" s="22" t="s">
+        <v>90</v>
+      </c>
+      <c r="H10" s="22" t="s">
+        <v>384</v>
+      </c>
+      <c r="I10" s="19" t="s">
+        <v>390</v>
+      </c>
     </row>
     <row r="11" spans="1:9" ht="66" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="28">
+      <c r="A11" s="23">
         <v>7</v>
       </c>
-      <c r="B11" s="22" t="s">
+      <c r="B11" s="17" t="s">
         <v>101</v>
       </c>
-      <c r="C11" s="28" t="s">
+      <c r="C11" s="23" t="s">
         <v>105</v>
       </c>
-      <c r="D11" s="22" t="s">
+      <c r="D11" s="17" t="s">
         <v>106</v>
       </c>
-      <c r="E11" s="22" t="s">
+      <c r="E11" s="17" t="s">
         <v>107</v>
       </c>
-      <c r="F11" s="34" t="s">
-        <v>90</v>
-      </c>
-      <c r="G11" s="28" t="s">
-        <v>90</v>
-      </c>
-      <c r="H11" s="28" t="s">
-        <v>86</v>
-      </c>
-      <c r="I11" s="22"/>
+      <c r="F11" s="29" t="s">
+        <v>90</v>
+      </c>
+      <c r="G11" s="23" t="s">
+        <v>90</v>
+      </c>
+      <c r="H11" s="23" t="s">
+        <v>384</v>
+      </c>
+      <c r="I11" s="17" t="s">
+        <v>391</v>
+      </c>
     </row>
     <row r="12" spans="1:9" ht="51" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="26">
+      <c r="A12" s="21">
         <v>8</v>
       </c>
-      <c r="B12" s="23" t="s">
+      <c r="B12" s="18" t="s">
         <v>101</v>
       </c>
-      <c r="C12" s="26" t="s">
+      <c r="C12" s="21" t="s">
         <v>108</v>
       </c>
-      <c r="D12" s="23" t="s">
+      <c r="D12" s="18" t="s">
         <v>109</v>
       </c>
-      <c r="E12" s="23" t="s">
+      <c r="E12" s="18" t="s">
         <v>110</v>
       </c>
-      <c r="F12" s="32" t="s">
-        <v>90</v>
-      </c>
-      <c r="G12" s="26" t="s">
+      <c r="F12" s="27" t="s">
+        <v>90</v>
+      </c>
+      <c r="G12" s="21" t="s">
         <v>97</v>
       </c>
-      <c r="H12" s="26" t="s">
-        <v>86</v>
-      </c>
-      <c r="I12" s="23"/>
+      <c r="H12" s="21" t="s">
+        <v>384</v>
+      </c>
+      <c r="I12" s="18" t="s">
+        <v>392</v>
+      </c>
     </row>
     <row r="13" spans="1:9" ht="51" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="27">
+      <c r="A13" s="22">
         <v>9</v>
       </c>
-      <c r="B13" s="24" t="s">
+      <c r="B13" s="19" t="s">
         <v>111</v>
       </c>
-      <c r="C13" s="27" t="s">
+      <c r="C13" s="22" t="s">
         <v>112</v>
       </c>
-      <c r="D13" s="24" t="s">
+      <c r="D13" s="19" t="s">
         <v>113</v>
       </c>
-      <c r="E13" s="24" t="s">
+      <c r="E13" s="19" t="s">
         <v>114</v>
       </c>
-      <c r="F13" s="33" t="s">
+      <c r="F13" s="28" t="s">
         <v>85</v>
       </c>
-      <c r="G13" s="27" t="s">
+      <c r="G13" s="22" t="s">
         <v>85</v>
       </c>
-      <c r="H13" s="27" t="s">
-        <v>86</v>
-      </c>
-      <c r="I13" s="24"/>
+      <c r="H13" s="22" t="s">
+        <v>86</v>
+      </c>
+      <c r="I13" s="19"/>
     </row>
     <row r="14" spans="1:9" ht="81" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="28">
+      <c r="A14" s="23">
         <v>10</v>
       </c>
-      <c r="B14" s="22" t="s">
+      <c r="B14" s="17" t="s">
         <v>111</v>
       </c>
-      <c r="C14" s="28" t="s">
+      <c r="C14" s="23" t="s">
         <v>115</v>
       </c>
-      <c r="D14" s="22" t="s">
+      <c r="D14" s="17" t="s">
         <v>116</v>
       </c>
-      <c r="E14" s="22" t="s">
+      <c r="E14" s="17" t="s">
         <v>117</v>
       </c>
-      <c r="F14" s="35" t="s">
+      <c r="F14" s="30" t="s">
         <v>84</v>
       </c>
-      <c r="G14" s="28" t="s">
+      <c r="G14" s="23" t="s">
         <v>85</v>
       </c>
-      <c r="H14" s="28" t="s">
-        <v>86</v>
-      </c>
-      <c r="I14" s="22"/>
+      <c r="H14" s="23" t="s">
+        <v>384</v>
+      </c>
+      <c r="I14" s="17" t="s">
+        <v>393</v>
+      </c>
     </row>
     <row r="15" spans="1:9" ht="51" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="25">
+      <c r="A15" s="20">
         <v>11</v>
       </c>
-      <c r="B15" s="7" t="s">
+      <c r="B15" s="12" t="s">
         <v>111</v>
       </c>
-      <c r="C15" s="25" t="s">
+      <c r="C15" s="20" t="s">
         <v>118</v>
       </c>
-      <c r="D15" s="7" t="s">
+      <c r="D15" s="12" t="s">
         <v>119</v>
       </c>
-      <c r="E15" s="7" t="s">
+      <c r="E15" s="12" t="s">
         <v>120</v>
       </c>
-      <c r="F15" s="31" t="s">
-        <v>90</v>
-      </c>
-      <c r="G15" s="25" t="s">
-        <v>90</v>
-      </c>
-      <c r="H15" s="25" t="s">
-        <v>86</v>
-      </c>
-      <c r="I15" s="7"/>
+      <c r="F15" s="26" t="s">
+        <v>90</v>
+      </c>
+      <c r="G15" s="20" t="s">
+        <v>90</v>
+      </c>
+      <c r="H15" s="20" t="s">
+        <v>86</v>
+      </c>
+      <c r="I15" s="12"/>
     </row>
     <row r="16" spans="1:9" ht="51" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="26">
+      <c r="A16" s="21">
         <v>12</v>
       </c>
-      <c r="B16" s="23" t="s">
+      <c r="B16" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="C16" s="26" t="s">
+      <c r="C16" s="21" t="s">
         <v>121</v>
       </c>
-      <c r="D16" s="23" t="s">
+      <c r="D16" s="18" t="s">
         <v>122</v>
       </c>
-      <c r="E16" s="23" t="s">
+      <c r="E16" s="18" t="s">
         <v>123</v>
       </c>
-      <c r="F16" s="32" t="s">
-        <v>90</v>
-      </c>
-      <c r="G16" s="26" t="s">
-        <v>90</v>
-      </c>
-      <c r="H16" s="26" t="s">
-        <v>86</v>
-      </c>
-      <c r="I16" s="23"/>
+      <c r="F16" s="27" t="s">
+        <v>90</v>
+      </c>
+      <c r="G16" s="21" t="s">
+        <v>90</v>
+      </c>
+      <c r="H16" s="21" t="s">
+        <v>86</v>
+      </c>
+      <c r="I16" s="18"/>
     </row>
     <row r="17" spans="1:9" ht="66" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="27">
+      <c r="A17" s="22">
         <v>13</v>
       </c>
-      <c r="B17" s="24" t="s">
+      <c r="B17" s="19" t="s">
         <v>124</v>
       </c>
-      <c r="C17" s="27" t="s">
+      <c r="C17" s="22" t="s">
         <v>125</v>
       </c>
-      <c r="D17" s="24" t="s">
+      <c r="D17" s="19" t="s">
         <v>126</v>
       </c>
-      <c r="E17" s="24" t="s">
+      <c r="E17" s="19" t="s">
         <v>127</v>
       </c>
-      <c r="F17" s="36" t="s">
-        <v>90</v>
-      </c>
-      <c r="G17" s="27" t="s">
+      <c r="F17" s="31" t="s">
+        <v>90</v>
+      </c>
+      <c r="G17" s="22" t="s">
         <v>97</v>
       </c>
-      <c r="H17" s="27" t="s">
-        <v>86</v>
-      </c>
-      <c r="I17" s="24"/>
+      <c r="H17" s="22" t="s">
+        <v>86</v>
+      </c>
+      <c r="I17" s="19"/>
     </row>
     <row r="18" spans="1:9" ht="51" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="29">
+      <c r="A18" s="24">
         <v>14</v>
       </c>
-      <c r="B18" s="21" t="s">
+      <c r="B18" s="16" t="s">
         <v>124</v>
       </c>
-      <c r="C18" s="29" t="s">
+      <c r="C18" s="24" t="s">
         <v>128</v>
       </c>
-      <c r="D18" s="21" t="s">
+      <c r="D18" s="16" t="s">
         <v>129</v>
       </c>
-      <c r="E18" s="21" t="s">
+      <c r="E18" s="16" t="s">
         <v>130</v>
       </c>
-      <c r="F18" s="37" t="s">
-        <v>90</v>
-      </c>
-      <c r="G18" s="29" t="s">
-        <v>90</v>
-      </c>
-      <c r="H18" s="29" t="s">
-        <v>86</v>
-      </c>
-      <c r="I18" s="21"/>
+      <c r="F18" s="32" t="s">
+        <v>90</v>
+      </c>
+      <c r="G18" s="24" t="s">
+        <v>90</v>
+      </c>
+      <c r="H18" s="24" t="s">
+        <v>86</v>
+      </c>
+      <c r="I18" s="16"/>
     </row>
     <row r="19" spans="1:9" ht="51" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="27">
+      <c r="A19" s="22">
         <v>15</v>
       </c>
-      <c r="B19" s="24" t="s">
+      <c r="B19" s="19" t="s">
         <v>131</v>
       </c>
-      <c r="C19" s="27" t="s">
+      <c r="C19" s="22" t="s">
         <v>132</v>
       </c>
-      <c r="D19" s="24" t="s">
+      <c r="D19" s="19" t="s">
         <v>133</v>
       </c>
-      <c r="E19" s="24" t="s">
+      <c r="E19" s="19" t="s">
         <v>134</v>
       </c>
-      <c r="F19" s="33" t="s">
+      <c r="F19" s="28" t="s">
         <v>85</v>
       </c>
-      <c r="G19" s="27" t="s">
+      <c r="G19" s="22" t="s">
         <v>85</v>
       </c>
-      <c r="H19" s="27" t="s">
-        <v>86</v>
-      </c>
-      <c r="I19" s="24"/>
+      <c r="H19" s="22" t="s">
+        <v>86</v>
+      </c>
+      <c r="I19" s="19"/>
     </row>
     <row r="20" spans="1:9" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="28">
+      <c r="A20" s="23">
         <v>16</v>
       </c>
-      <c r="B20" s="22" t="s">
+      <c r="B20" s="17" t="s">
         <v>131</v>
       </c>
-      <c r="C20" s="28" t="s">
+      <c r="C20" s="23" t="s">
         <v>135</v>
       </c>
-      <c r="D20" s="22" t="s">
+      <c r="D20" s="17" t="s">
         <v>136</v>
       </c>
-      <c r="E20" s="22" t="s">
+      <c r="E20" s="17" t="s">
         <v>137</v>
       </c>
-      <c r="F20" s="34" t="s">
-        <v>90</v>
-      </c>
-      <c r="G20" s="28" t="s">
-        <v>90</v>
-      </c>
-      <c r="H20" s="28" t="s">
-        <v>86</v>
-      </c>
-      <c r="I20" s="22"/>
+      <c r="F20" s="29" t="s">
+        <v>90</v>
+      </c>
+      <c r="G20" s="23" t="s">
+        <v>90</v>
+      </c>
+      <c r="H20" s="23" t="s">
+        <v>86</v>
+      </c>
+      <c r="I20" s="17"/>
     </row>
     <row r="21" spans="1:9" ht="36" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="26">
+      <c r="A21" s="21">
         <v>17</v>
       </c>
-      <c r="B21" s="23" t="s">
+      <c r="B21" s="18" t="s">
         <v>131</v>
       </c>
-      <c r="C21" s="26" t="s">
+      <c r="C21" s="21" t="s">
         <v>138</v>
       </c>
-      <c r="D21" s="23" t="s">
+      <c r="D21" s="18" t="s">
         <v>139</v>
       </c>
-      <c r="E21" s="23" t="s">
+      <c r="E21" s="18" t="s">
         <v>140</v>
       </c>
-      <c r="F21" s="32" t="s">
-        <v>90</v>
-      </c>
-      <c r="G21" s="26" t="s">
-        <v>90</v>
-      </c>
-      <c r="H21" s="26" t="s">
-        <v>86</v>
-      </c>
-      <c r="I21" s="23"/>
+      <c r="F21" s="27" t="s">
+        <v>90</v>
+      </c>
+      <c r="G21" s="21" t="s">
+        <v>90</v>
+      </c>
+      <c r="H21" s="21" t="s">
+        <v>86</v>
+      </c>
+      <c r="I21" s="18"/>
     </row>
     <row r="22" spans="1:9" ht="51" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="27">
+      <c r="A22" s="22">
         <v>18</v>
       </c>
-      <c r="B22" s="24" t="s">
+      <c r="B22" s="19" t="s">
         <v>141</v>
       </c>
-      <c r="C22" s="27" t="s">
+      <c r="C22" s="22" t="s">
         <v>142</v>
       </c>
-      <c r="D22" s="24" t="s">
+      <c r="D22" s="19" t="s">
         <v>143</v>
       </c>
-      <c r="E22" s="24" t="s">
+      <c r="E22" s="19" t="s">
         <v>144</v>
       </c>
-      <c r="F22" s="36" t="s">
-        <v>90</v>
-      </c>
-      <c r="G22" s="27" t="s">
+      <c r="F22" s="31" t="s">
+        <v>90</v>
+      </c>
+      <c r="G22" s="22" t="s">
         <v>85</v>
       </c>
-      <c r="H22" s="27" t="s">
-        <v>86</v>
-      </c>
-      <c r="I22" s="24"/>
+      <c r="H22" s="22" t="s">
+        <v>86</v>
+      </c>
+      <c r="I22" s="19"/>
     </row>
     <row r="23" spans="1:9" ht="51" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="28">
+      <c r="A23" s="23">
         <v>19</v>
       </c>
-      <c r="B23" s="22" t="s">
+      <c r="B23" s="17" t="s">
         <v>141</v>
       </c>
-      <c r="C23" s="28" t="s">
+      <c r="C23" s="23" t="s">
         <v>145</v>
       </c>
-      <c r="D23" s="22" t="s">
+      <c r="D23" s="17" t="s">
         <v>146</v>
       </c>
-      <c r="E23" s="22" t="s">
+      <c r="E23" s="17" t="s">
         <v>147</v>
       </c>
-      <c r="F23" s="34" t="s">
-        <v>90</v>
-      </c>
-      <c r="G23" s="28" t="s">
-        <v>90</v>
-      </c>
-      <c r="H23" s="28" t="s">
-        <v>86</v>
-      </c>
-      <c r="I23" s="22"/>
+      <c r="F23" s="29" t="s">
+        <v>90</v>
+      </c>
+      <c r="G23" s="23" t="s">
+        <v>90</v>
+      </c>
+      <c r="H23" s="23" t="s">
+        <v>86</v>
+      </c>
+      <c r="I23" s="17"/>
     </row>
     <row r="24" spans="1:9" ht="51" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="25">
+      <c r="A24" s="20">
         <v>20</v>
       </c>
-      <c r="B24" s="7" t="s">
+      <c r="B24" s="12" t="s">
         <v>141</v>
       </c>
-      <c r="C24" s="25" t="s">
+      <c r="C24" s="20" t="s">
         <v>148</v>
       </c>
-      <c r="D24" s="7" t="s">
+      <c r="D24" s="12" t="s">
         <v>149</v>
       </c>
-      <c r="E24" s="7" t="s">
+      <c r="E24" s="12" t="s">
         <v>150</v>
       </c>
-      <c r="F24" s="31" t="s">
-        <v>90</v>
-      </c>
-      <c r="G24" s="25" t="s">
-        <v>90</v>
-      </c>
-      <c r="H24" s="25" t="s">
-        <v>86</v>
-      </c>
-      <c r="I24" s="7"/>
+      <c r="F24" s="26" t="s">
+        <v>90</v>
+      </c>
+      <c r="G24" s="20" t="s">
+        <v>90</v>
+      </c>
+      <c r="H24" s="20" t="s">
+        <v>86</v>
+      </c>
+      <c r="I24" s="12"/>
     </row>
     <row r="25" spans="1:9" ht="51" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="25">
+      <c r="A25" s="20">
         <v>21</v>
       </c>
-      <c r="B25" s="7" t="s">
+      <c r="B25" s="12" t="s">
         <v>141</v>
       </c>
-      <c r="C25" s="25" t="s">
+      <c r="C25" s="20" t="s">
         <v>151</v>
       </c>
-      <c r="D25" s="7" t="s">
+      <c r="D25" s="12" t="s">
         <v>152</v>
       </c>
-      <c r="E25" s="7" t="s">
+      <c r="E25" s="12" t="s">
         <v>153</v>
       </c>
-      <c r="F25" s="31" t="s">
-        <v>90</v>
-      </c>
-      <c r="G25" s="25" t="s">
-        <v>90</v>
-      </c>
-      <c r="H25" s="25" t="s">
-        <v>86</v>
-      </c>
-      <c r="I25" s="7"/>
+      <c r="F25" s="26" t="s">
+        <v>90</v>
+      </c>
+      <c r="G25" s="20" t="s">
+        <v>90</v>
+      </c>
+      <c r="H25" s="20" t="s">
+        <v>86</v>
+      </c>
+      <c r="I25" s="12"/>
     </row>
     <row r="26" spans="1:9" ht="51" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="25">
+      <c r="A26" s="20">
         <v>22</v>
       </c>
-      <c r="B26" s="7" t="s">
+      <c r="B26" s="12" t="s">
         <v>141</v>
       </c>
-      <c r="C26" s="25" t="s">
+      <c r="C26" s="20" t="s">
         <v>154</v>
       </c>
-      <c r="D26" s="7" t="s">
+      <c r="D26" s="12" t="s">
         <v>155</v>
       </c>
-      <c r="E26" s="7" t="s">
+      <c r="E26" s="12" t="s">
         <v>156</v>
       </c>
-      <c r="F26" s="31" t="s">
-        <v>90</v>
-      </c>
-      <c r="G26" s="25" t="s">
+      <c r="F26" s="26" t="s">
+        <v>90</v>
+      </c>
+      <c r="G26" s="20" t="s">
         <v>97</v>
       </c>
-      <c r="H26" s="25" t="s">
-        <v>86</v>
-      </c>
-      <c r="I26" s="7"/>
+      <c r="H26" s="20" t="s">
+        <v>86</v>
+      </c>
+      <c r="I26" s="12"/>
     </row>
     <row r="27" spans="1:9" ht="51" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="26">
+      <c r="A27" s="21">
         <v>23</v>
       </c>
-      <c r="B27" s="23" t="s">
+      <c r="B27" s="18" t="s">
         <v>141</v>
       </c>
-      <c r="C27" s="26" t="s">
+      <c r="C27" s="21" t="s">
         <v>157</v>
       </c>
-      <c r="D27" s="23" t="s">
+      <c r="D27" s="18" t="s">
         <v>158</v>
       </c>
-      <c r="E27" s="23" t="s">
+      <c r="E27" s="18" t="s">
         <v>159</v>
       </c>
-      <c r="F27" s="32" t="s">
-        <v>90</v>
-      </c>
-      <c r="G27" s="26" t="s">
+      <c r="F27" s="27" t="s">
+        <v>90</v>
+      </c>
+      <c r="G27" s="21" t="s">
         <v>97</v>
       </c>
-      <c r="H27" s="26" t="s">
-        <v>86</v>
-      </c>
-      <c r="I27" s="23"/>
+      <c r="H27" s="21" t="s">
+        <v>86</v>
+      </c>
+      <c r="I27" s="18"/>
     </row>
     <row r="28" spans="1:9" ht="66" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="27">
+      <c r="A28" s="22">
         <v>24</v>
       </c>
-      <c r="B28" s="24" t="s">
+      <c r="B28" s="19" t="s">
         <v>160</v>
       </c>
-      <c r="C28" s="27" t="s">
+      <c r="C28" s="22" t="s">
         <v>161</v>
       </c>
-      <c r="D28" s="24" t="s">
+      <c r="D28" s="19" t="s">
         <v>162</v>
       </c>
-      <c r="E28" s="24" t="s">
+      <c r="E28" s="19" t="s">
         <v>163</v>
       </c>
-      <c r="F28" s="38" t="s">
+      <c r="F28" s="33" t="s">
         <v>84</v>
       </c>
-      <c r="G28" s="27" t="s">
+      <c r="G28" s="22" t="s">
         <v>85</v>
       </c>
-      <c r="H28" s="27" t="s">
-        <v>86</v>
-      </c>
-      <c r="I28" s="24"/>
+      <c r="H28" s="22" t="s">
+        <v>384</v>
+      </c>
+      <c r="I28" s="19" t="s">
+        <v>394</v>
+      </c>
     </row>
     <row r="29" spans="1:9" ht="66" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="28">
+      <c r="A29" s="23">
         <v>25</v>
       </c>
-      <c r="B29" s="22" t="s">
+      <c r="B29" s="17" t="s">
         <v>160</v>
       </c>
-      <c r="C29" s="28" t="s">
+      <c r="C29" s="23" t="s">
         <v>164</v>
       </c>
-      <c r="D29" s="22" t="s">
+      <c r="D29" s="17" t="s">
         <v>165</v>
       </c>
-      <c r="E29" s="22" t="s">
+      <c r="E29" s="17" t="s">
         <v>166</v>
       </c>
-      <c r="F29" s="35" t="s">
+      <c r="F29" s="30" t="s">
         <v>84</v>
       </c>
-      <c r="G29" s="28" t="s">
+      <c r="G29" s="23" t="s">
         <v>85</v>
       </c>
-      <c r="H29" s="28" t="s">
-        <v>86</v>
-      </c>
-      <c r="I29" s="22"/>
+      <c r="H29" s="23" t="s">
+        <v>384</v>
+      </c>
+      <c r="I29" s="17" t="s">
+        <v>395</v>
+      </c>
     </row>
     <row r="30" spans="1:9" ht="66" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="25">
+      <c r="A30" s="20">
         <v>26</v>
       </c>
-      <c r="B30" s="7" t="s">
+      <c r="B30" s="12" t="s">
         <v>160</v>
       </c>
-      <c r="C30" s="25" t="s">
+      <c r="C30" s="20" t="s">
         <v>167</v>
       </c>
-      <c r="D30" s="7" t="s">
+      <c r="D30" s="12" t="s">
         <v>168</v>
       </c>
-      <c r="E30" s="7" t="s">
+      <c r="E30" s="12" t="s">
         <v>169</v>
       </c>
-      <c r="F30" s="30" t="s">
+      <c r="F30" s="25" t="s">
         <v>84</v>
       </c>
-      <c r="G30" s="25" t="s">
+      <c r="G30" s="20" t="s">
         <v>85</v>
       </c>
-      <c r="H30" s="25" t="s">
-        <v>86</v>
-      </c>
-      <c r="I30" s="7"/>
+      <c r="H30" s="20" t="s">
+        <v>384</v>
+      </c>
+      <c r="I30" s="12" t="s">
+        <v>396</v>
+      </c>
     </row>
     <row r="31" spans="1:9" ht="51" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="26">
+      <c r="A31" s="21">
         <v>27</v>
       </c>
-      <c r="B31" s="23" t="s">
+      <c r="B31" s="18" t="s">
         <v>160</v>
       </c>
-      <c r="C31" s="26" t="s">
+      <c r="C31" s="21" t="s">
         <v>170</v>
       </c>
-      <c r="D31" s="23" t="s">
+      <c r="D31" s="18" t="s">
         <v>171</v>
       </c>
-      <c r="E31" s="23" t="s">
+      <c r="E31" s="18" t="s">
         <v>172</v>
       </c>
-      <c r="F31" s="32" t="s">
-        <v>90</v>
-      </c>
-      <c r="G31" s="26" t="s">
-        <v>90</v>
-      </c>
-      <c r="H31" s="26" t="s">
-        <v>86</v>
-      </c>
-      <c r="I31" s="23"/>
+      <c r="F31" s="27" t="s">
+        <v>90</v>
+      </c>
+      <c r="G31" s="21" t="s">
+        <v>90</v>
+      </c>
+      <c r="H31" s="21" t="s">
+        <v>384</v>
+      </c>
+      <c r="I31" s="18" t="s">
+        <v>397</v>
+      </c>
     </row>
     <row r="32" spans="1:9" ht="66" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="27">
+      <c r="A32" s="22">
         <v>28</v>
       </c>
-      <c r="B32" s="24" t="s">
+      <c r="B32" s="19" t="s">
         <v>173</v>
       </c>
-      <c r="C32" s="27" t="s">
+      <c r="C32" s="22" t="s">
         <v>174</v>
       </c>
-      <c r="D32" s="24" t="s">
+      <c r="D32" s="19" t="s">
         <v>175</v>
       </c>
-      <c r="E32" s="24" t="s">
+      <c r="E32" s="19" t="s">
         <v>176</v>
       </c>
-      <c r="F32" s="36" t="s">
-        <v>90</v>
-      </c>
-      <c r="G32" s="27" t="s">
-        <v>90</v>
-      </c>
-      <c r="H32" s="27" t="s">
-        <v>86</v>
-      </c>
-      <c r="I32" s="24"/>
+      <c r="F32" s="31" t="s">
+        <v>90</v>
+      </c>
+      <c r="G32" s="22" t="s">
+        <v>90</v>
+      </c>
+      <c r="H32" s="22" t="s">
+        <v>86</v>
+      </c>
+      <c r="I32" s="19"/>
     </row>
     <row r="33" spans="1:9" ht="81" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="28">
+      <c r="A33" s="23">
         <v>29</v>
       </c>
-      <c r="B33" s="22" t="s">
+      <c r="B33" s="17" t="s">
         <v>173</v>
       </c>
-      <c r="C33" s="28" t="s">
+      <c r="C33" s="23" t="s">
         <v>177</v>
       </c>
-      <c r="D33" s="22" t="s">
+      <c r="D33" s="17" t="s">
         <v>178</v>
       </c>
-      <c r="E33" s="22" t="s">
+      <c r="E33" s="17" t="s">
         <v>179</v>
       </c>
-      <c r="F33" s="34" t="s">
-        <v>90</v>
-      </c>
-      <c r="G33" s="28" t="s">
-        <v>90</v>
-      </c>
-      <c r="H33" s="28" t="s">
-        <v>86</v>
-      </c>
-      <c r="I33" s="22"/>
+      <c r="F33" s="29" t="s">
+        <v>90</v>
+      </c>
+      <c r="G33" s="23" t="s">
+        <v>90</v>
+      </c>
+      <c r="H33" s="23" t="s">
+        <v>86</v>
+      </c>
+      <c r="I33" s="17"/>
     </row>
     <row r="34" spans="1:9" ht="51" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="25">
+      <c r="A34" s="20">
         <v>30</v>
       </c>
-      <c r="B34" s="7" t="s">
+      <c r="B34" s="12" t="s">
         <v>173</v>
       </c>
-      <c r="C34" s="25" t="s">
+      <c r="C34" s="20" t="s">
         <v>180</v>
       </c>
-      <c r="D34" s="7" t="s">
+      <c r="D34" s="12" t="s">
         <v>181</v>
       </c>
-      <c r="E34" s="7" t="s">
+      <c r="E34" s="12" t="s">
         <v>182</v>
       </c>
-      <c r="F34" s="31" t="s">
-        <v>90</v>
-      </c>
-      <c r="G34" s="25" t="s">
-        <v>90</v>
-      </c>
-      <c r="H34" s="25" t="s">
-        <v>86</v>
-      </c>
-      <c r="I34" s="7"/>
+      <c r="F34" s="26" t="s">
+        <v>90</v>
+      </c>
+      <c r="G34" s="20" t="s">
+        <v>90</v>
+      </c>
+      <c r="H34" s="20" t="s">
+        <v>86</v>
+      </c>
+      <c r="I34" s="12"/>
     </row>
     <row r="35" spans="1:9" ht="66" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="25">
+      <c r="A35" s="20">
         <v>31</v>
       </c>
-      <c r="B35" s="7" t="s">
+      <c r="B35" s="12" t="s">
         <v>173</v>
       </c>
-      <c r="C35" s="25" t="s">
+      <c r="C35" s="20" t="s">
         <v>183</v>
       </c>
-      <c r="D35" s="7" t="s">
+      <c r="D35" s="12" t="s">
         <v>184</v>
       </c>
-      <c r="E35" s="7" t="s">
+      <c r="E35" s="12" t="s">
         <v>185</v>
       </c>
-      <c r="F35" s="31" t="s">
-        <v>90</v>
-      </c>
-      <c r="G35" s="25" t="s">
-        <v>90</v>
-      </c>
-      <c r="H35" s="25" t="s">
-        <v>86</v>
-      </c>
-      <c r="I35" s="7"/>
+      <c r="F35" s="26" t="s">
+        <v>90</v>
+      </c>
+      <c r="G35" s="20" t="s">
+        <v>90</v>
+      </c>
+      <c r="H35" s="20" t="s">
+        <v>86</v>
+      </c>
+      <c r="I35" s="12"/>
     </row>
     <row r="36" spans="1:9" ht="51" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="25">
+      <c r="A36" s="20">
         <v>32</v>
       </c>
-      <c r="B36" s="7" t="s">
+      <c r="B36" s="12" t="s">
         <v>173</v>
       </c>
-      <c r="C36" s="25" t="s">
+      <c r="C36" s="20" t="s">
         <v>186</v>
       </c>
-      <c r="D36" s="7" t="s">
+      <c r="D36" s="12" t="s">
         <v>187</v>
       </c>
-      <c r="E36" s="7" t="s">
+      <c r="E36" s="12" t="s">
         <v>188</v>
       </c>
-      <c r="F36" s="31" t="s">
-        <v>90</v>
-      </c>
-      <c r="G36" s="25" t="s">
+      <c r="F36" s="26" t="s">
+        <v>90</v>
+      </c>
+      <c r="G36" s="20" t="s">
         <v>97</v>
       </c>
-      <c r="H36" s="25" t="s">
-        <v>86</v>
-      </c>
-      <c r="I36" s="7"/>
+      <c r="H36" s="20" t="s">
+        <v>86</v>
+      </c>
+      <c r="I36" s="12"/>
     </row>
     <row r="37" spans="1:9" ht="51" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="26">
+      <c r="A37" s="21">
         <v>33</v>
       </c>
-      <c r="B37" s="23" t="s">
+      <c r="B37" s="18" t="s">
         <v>173</v>
       </c>
-      <c r="C37" s="26" t="s">
+      <c r="C37" s="21" t="s">
         <v>189</v>
       </c>
-      <c r="D37" s="23" t="s">
+      <c r="D37" s="18" t="s">
         <v>190</v>
       </c>
-      <c r="E37" s="23" t="s">
+      <c r="E37" s="18" t="s">
         <v>191</v>
       </c>
-      <c r="F37" s="32" t="s">
-        <v>90</v>
-      </c>
-      <c r="G37" s="26" t="s">
+      <c r="F37" s="27" t="s">
+        <v>90</v>
+      </c>
+      <c r="G37" s="21" t="s">
         <v>97</v>
       </c>
-      <c r="H37" s="26" t="s">
-        <v>86</v>
-      </c>
-      <c r="I37" s="23"/>
+      <c r="H37" s="21" t="s">
+        <v>86</v>
+      </c>
+      <c r="I37" s="18"/>
     </row>
     <row r="38" spans="1:9" ht="51" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="27">
+      <c r="A38" s="22">
         <v>34</v>
       </c>
-      <c r="B38" s="24" t="s">
+      <c r="B38" s="19" t="s">
         <v>192</v>
       </c>
-      <c r="C38" s="27" t="s">
+      <c r="C38" s="22" t="s">
         <v>193</v>
       </c>
-      <c r="D38" s="24" t="s">
+      <c r="D38" s="19" t="s">
         <v>194</v>
       </c>
-      <c r="E38" s="24" t="s">
+      <c r="E38" s="19" t="s">
         <v>195</v>
       </c>
-      <c r="F38" s="33" t="s">
+      <c r="F38" s="28" t="s">
         <v>85</v>
       </c>
-      <c r="G38" s="27" t="s">
+      <c r="G38" s="22" t="s">
         <v>85</v>
       </c>
-      <c r="H38" s="27" t="s">
-        <v>86</v>
-      </c>
-      <c r="I38" s="24"/>
+      <c r="H38" s="22" t="s">
+        <v>384</v>
+      </c>
+      <c r="I38" s="19" t="s">
+        <v>398</v>
+      </c>
     </row>
     <row r="39" spans="1:9" ht="66" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="28">
+      <c r="A39" s="23">
         <v>35</v>
       </c>
-      <c r="B39" s="22" t="s">
+      <c r="B39" s="17" t="s">
         <v>192</v>
       </c>
-      <c r="C39" s="28" t="s">
+      <c r="C39" s="23" t="s">
         <v>196</v>
       </c>
-      <c r="D39" s="22" t="s">
+      <c r="D39" s="17" t="s">
         <v>197</v>
       </c>
-      <c r="E39" s="22" t="s">
+      <c r="E39" s="17" t="s">
         <v>198</v>
       </c>
-      <c r="F39" s="39" t="s">
+      <c r="F39" s="34" t="s">
         <v>85</v>
       </c>
-      <c r="G39" s="28" t="s">
+      <c r="G39" s="23" t="s">
         <v>85</v>
       </c>
-      <c r="H39" s="28" t="s">
-        <v>86</v>
-      </c>
-      <c r="I39" s="22"/>
+      <c r="H39" s="23" t="s">
+        <v>384</v>
+      </c>
+      <c r="I39" s="17" t="s">
+        <v>399</v>
+      </c>
     </row>
     <row r="40" spans="1:9" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="25">
+      <c r="A40" s="20">
         <v>36</v>
       </c>
-      <c r="B40" s="7" t="s">
+      <c r="B40" s="12" t="s">
         <v>192</v>
       </c>
-      <c r="C40" s="25" t="s">
+      <c r="C40" s="20" t="s">
         <v>199</v>
       </c>
-      <c r="D40" s="7" t="s">
+      <c r="D40" s="12" t="s">
         <v>200</v>
       </c>
-      <c r="E40" s="7" t="s">
+      <c r="E40" s="12" t="s">
         <v>201</v>
       </c>
-      <c r="F40" s="31" t="s">
-        <v>90</v>
-      </c>
-      <c r="G40" s="25" t="s">
+      <c r="F40" s="26" t="s">
+        <v>90</v>
+      </c>
+      <c r="G40" s="20" t="s">
         <v>97</v>
       </c>
-      <c r="H40" s="25" t="s">
-        <v>86</v>
-      </c>
-      <c r="I40" s="7"/>
+      <c r="H40" s="20" t="s">
+        <v>384</v>
+      </c>
+      <c r="I40" s="12" t="s">
+        <v>400</v>
+      </c>
     </row>
     <row r="41" spans="1:9" ht="51" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="26">
+      <c r="A41" s="21">
         <v>37</v>
       </c>
-      <c r="B41" s="23" t="s">
+      <c r="B41" s="18" t="s">
         <v>192</v>
       </c>
-      <c r="C41" s="26" t="s">
+      <c r="C41" s="21" t="s">
         <v>202</v>
       </c>
-      <c r="D41" s="23" t="s">
+      <c r="D41" s="18" t="s">
         <v>203</v>
       </c>
-      <c r="E41" s="23" t="s">
+      <c r="E41" s="18" t="s">
         <v>204</v>
       </c>
-      <c r="F41" s="32" t="s">
-        <v>90</v>
-      </c>
-      <c r="G41" s="26" t="s">
+      <c r="F41" s="27" t="s">
+        <v>90</v>
+      </c>
+      <c r="G41" s="21" t="s">
         <v>97</v>
       </c>
-      <c r="H41" s="26" t="s">
-        <v>86</v>
-      </c>
-      <c r="I41" s="23"/>
+      <c r="H41" s="21" t="s">
+        <v>384</v>
+      </c>
+      <c r="I41" s="18" t="s">
+        <v>401</v>
+      </c>
     </row>
     <row r="42" spans="1:9" ht="51" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="27">
+      <c r="A42" s="22">
         <v>38</v>
       </c>
-      <c r="B42" s="24" t="s">
+      <c r="B42" s="19" t="s">
         <v>205</v>
       </c>
-      <c r="C42" s="27" t="s">
+      <c r="C42" s="22" t="s">
         <v>206</v>
       </c>
-      <c r="D42" s="24" t="s">
+      <c r="D42" s="19" t="s">
         <v>207</v>
       </c>
-      <c r="E42" s="24" t="s">
+      <c r="E42" s="19" t="s">
         <v>208</v>
       </c>
-      <c r="F42" s="38" t="s">
+      <c r="F42" s="33" t="s">
         <v>84</v>
       </c>
-      <c r="G42" s="27" t="s">
+      <c r="G42" s="22" t="s">
         <v>85</v>
       </c>
-      <c r="H42" s="27" t="s">
-        <v>86</v>
-      </c>
-      <c r="I42" s="24"/>
+      <c r="H42" s="22" t="s">
+        <v>384</v>
+      </c>
+      <c r="I42" s="19" t="s">
+        <v>402</v>
+      </c>
     </row>
     <row r="43" spans="1:9" ht="51" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="28">
+      <c r="A43" s="23">
         <v>39</v>
       </c>
-      <c r="B43" s="22" t="s">
+      <c r="B43" s="17" t="s">
         <v>205</v>
       </c>
-      <c r="C43" s="28" t="s">
+      <c r="C43" s="23" t="s">
         <v>209</v>
       </c>
-      <c r="D43" s="22" t="s">
+      <c r="D43" s="17" t="s">
         <v>210</v>
       </c>
-      <c r="E43" s="22" t="s">
+      <c r="E43" s="17" t="s">
         <v>211</v>
       </c>
-      <c r="F43" s="39" t="s">
+      <c r="F43" s="34" t="s">
         <v>85</v>
       </c>
-      <c r="G43" s="28" t="s">
+      <c r="G43" s="23" t="s">
         <v>85</v>
       </c>
-      <c r="H43" s="28" t="s">
-        <v>86</v>
-      </c>
-      <c r="I43" s="22"/>
+      <c r="H43" s="23" t="s">
+        <v>384</v>
+      </c>
+      <c r="I43" s="17" t="s">
+        <v>403</v>
+      </c>
     </row>
     <row r="44" spans="1:9" ht="51" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="25">
+      <c r="A44" s="20">
         <v>40</v>
       </c>
-      <c r="B44" s="7" t="s">
+      <c r="B44" s="12" t="s">
         <v>205</v>
       </c>
-      <c r="C44" s="25" t="s">
+      <c r="C44" s="20" t="s">
         <v>212</v>
       </c>
-      <c r="D44" s="7" t="s">
+      <c r="D44" s="12" t="s">
         <v>213</v>
       </c>
-      <c r="E44" s="7" t="s">
+      <c r="E44" s="12" t="s">
         <v>214</v>
       </c>
-      <c r="F44" s="40" t="s">
+      <c r="F44" s="35" t="s">
         <v>85</v>
       </c>
-      <c r="G44" s="25" t="s">
+      <c r="G44" s="20" t="s">
         <v>85</v>
       </c>
-      <c r="H44" s="25" t="s">
-        <v>86</v>
-      </c>
-      <c r="I44" s="7"/>
+      <c r="H44" s="20" t="s">
+        <v>384</v>
+      </c>
+      <c r="I44" s="12" t="s">
+        <v>404</v>
+      </c>
     </row>
     <row r="45" spans="1:9" ht="51" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="25">
+      <c r="A45" s="20">
         <v>41</v>
       </c>
-      <c r="B45" s="7" t="s">
+      <c r="B45" s="12" t="s">
         <v>205</v>
       </c>
-      <c r="C45" s="25" t="s">
+      <c r="C45" s="20" t="s">
         <v>215</v>
       </c>
-      <c r="D45" s="7" t="s">
+      <c r="D45" s="12" t="s">
         <v>216</v>
       </c>
-      <c r="E45" s="7" t="s">
+      <c r="E45" s="12" t="s">
         <v>217</v>
       </c>
-      <c r="F45" s="31" t="s">
-        <v>90</v>
-      </c>
-      <c r="G45" s="25" t="s">
+      <c r="F45" s="26" t="s">
+        <v>90</v>
+      </c>
+      <c r="G45" s="20" t="s">
         <v>85</v>
       </c>
-      <c r="H45" s="25" t="s">
-        <v>86</v>
-      </c>
-      <c r="I45" s="7"/>
+      <c r="H45" s="20" t="s">
+        <v>384</v>
+      </c>
+      <c r="I45" s="12" t="s">
+        <v>405</v>
+      </c>
     </row>
     <row r="46" spans="1:9" ht="51" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="25">
+      <c r="A46" s="20">
         <v>42</v>
       </c>
-      <c r="B46" s="7" t="s">
+      <c r="B46" s="12" t="s">
         <v>205</v>
       </c>
-      <c r="C46" s="25" t="s">
+      <c r="C46" s="20" t="s">
         <v>218</v>
       </c>
-      <c r="D46" s="7" t="s">
+      <c r="D46" s="12" t="s">
         <v>219</v>
       </c>
-      <c r="E46" s="7" t="s">
+      <c r="E46" s="12" t="s">
         <v>220</v>
       </c>
-      <c r="F46" s="31" t="s">
-        <v>90</v>
-      </c>
-      <c r="G46" s="25" t="s">
+      <c r="F46" s="26" t="s">
+        <v>90</v>
+      </c>
+      <c r="G46" s="20" t="s">
         <v>85</v>
       </c>
-      <c r="H46" s="25" t="s">
-        <v>86</v>
-      </c>
-      <c r="I46" s="7"/>
+      <c r="H46" s="20" t="s">
+        <v>384</v>
+      </c>
+      <c r="I46" s="12" t="s">
+        <v>406</v>
+      </c>
     </row>
     <row r="47" spans="1:9" ht="66" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="25">
+      <c r="A47" s="20">
         <v>43</v>
       </c>
-      <c r="B47" s="7" t="s">
+      <c r="B47" s="12" t="s">
         <v>205</v>
       </c>
-      <c r="C47" s="25" t="s">
+      <c r="C47" s="20" t="s">
         <v>221</v>
       </c>
-      <c r="D47" s="7" t="s">
+      <c r="D47" s="12" t="s">
         <v>222</v>
       </c>
-      <c r="E47" s="7" t="s">
+      <c r="E47" s="12" t="s">
         <v>223</v>
       </c>
-      <c r="F47" s="31" t="s">
-        <v>90</v>
-      </c>
-      <c r="G47" s="25" t="s">
+      <c r="F47" s="26" t="s">
+        <v>90</v>
+      </c>
+      <c r="G47" s="20" t="s">
         <v>85</v>
       </c>
-      <c r="H47" s="25" t="s">
-        <v>86</v>
-      </c>
-      <c r="I47" s="7"/>
+      <c r="H47" s="20" t="s">
+        <v>384</v>
+      </c>
+      <c r="I47" s="12" t="s">
+        <v>407</v>
+      </c>
     </row>
     <row r="48" spans="1:9" ht="51" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="25">
+      <c r="A48" s="20">
         <v>44</v>
       </c>
-      <c r="B48" s="7" t="s">
+      <c r="B48" s="12" t="s">
         <v>205</v>
       </c>
-      <c r="C48" s="25" t="s">
+      <c r="C48" s="20" t="s">
         <v>224</v>
       </c>
-      <c r="D48" s="7" t="s">
+      <c r="D48" s="12" t="s">
         <v>225</v>
       </c>
-      <c r="E48" s="7" t="s">
+      <c r="E48" s="12" t="s">
         <v>226</v>
       </c>
-      <c r="F48" s="31" t="s">
-        <v>90</v>
-      </c>
-      <c r="G48" s="25" t="s">
-        <v>90</v>
-      </c>
-      <c r="H48" s="25" t="s">
-        <v>86</v>
-      </c>
-      <c r="I48" s="7"/>
+      <c r="F48" s="26" t="s">
+        <v>90</v>
+      </c>
+      <c r="G48" s="20" t="s">
+        <v>90</v>
+      </c>
+      <c r="H48" s="20" t="s">
+        <v>384</v>
+      </c>
+      <c r="I48" s="12" t="s">
+        <v>408</v>
+      </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
@@ -3747,7 +3870,7 @@
       </c>
       <c r="B50" s="2" t="str">
         <f>COUNTIF(H5:H48,"Corregido")&amp;" de 44 corregidos"</f>
-        <v>0 de 44 corregidos</v>
+        <v>24 de 44 corregidos</v>
       </c>
     </row>
   </sheetData>
@@ -3789,7 +3912,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:I22"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.7109375" customWidth="1"/>
     <col min="2" max="2" width="24.7109375" customWidth="1"/>
@@ -3807,478 +3930,478 @@
       </c>
     </row>
     <row r="2" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="20" t="s">
+      <c r="A2" s="39" t="s">
         <v>229</v>
       </c>
-      <c r="B2" s="20"/>
-      <c r="C2" s="20"/>
-      <c r="D2" s="20"/>
-      <c r="E2" s="20"/>
-      <c r="F2" s="20"/>
-      <c r="G2" s="20"/>
-      <c r="H2" s="20"/>
-      <c r="I2" s="20"/>
+      <c r="B2" s="39"/>
+      <c r="C2" s="39"/>
+      <c r="D2" s="39"/>
+      <c r="E2" s="39"/>
+      <c r="F2" s="39"/>
+      <c r="G2" s="39"/>
+      <c r="H2" s="39"/>
+      <c r="I2" s="39"/>
     </row>
     <row r="4" spans="1:9" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="11" t="s">
         <v>71</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="11" t="s">
         <v>73</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="11" t="s">
         <v>74</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="11" t="s">
         <v>75</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="F4" s="11" t="s">
         <v>76</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="G4" s="11" t="s">
         <v>77</v>
       </c>
-      <c r="H4" s="3" t="s">
+      <c r="H4" s="11" t="s">
         <v>78</v>
       </c>
-      <c r="I4" s="3" t="s">
+      <c r="I4" s="11" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="25">
+      <c r="A5" s="20">
         <v>1</v>
       </c>
-      <c r="B5" s="7" t="s">
+      <c r="B5" s="12" t="s">
         <v>51</v>
       </c>
-      <c r="C5" s="25" t="s">
+      <c r="C5" s="20" t="s">
         <v>230</v>
       </c>
-      <c r="D5" s="7" t="s">
+      <c r="D5" s="12" t="s">
         <v>231</v>
       </c>
-      <c r="E5" s="7" t="s">
+      <c r="E5" s="12" t="s">
         <v>232</v>
       </c>
-      <c r="F5" s="40" t="s">
+      <c r="F5" s="35" t="s">
         <v>85</v>
       </c>
-      <c r="G5" s="25" t="s">
+      <c r="G5" s="20" t="s">
         <v>85</v>
       </c>
-      <c r="H5" s="25" t="s">
-        <v>86</v>
-      </c>
-      <c r="I5" s="7"/>
+      <c r="H5" s="20" t="s">
+        <v>86</v>
+      </c>
+      <c r="I5" s="12"/>
     </row>
     <row r="6" spans="1:9" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="25">
+      <c r="A6" s="20">
         <v>2</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="B6" s="12" t="s">
         <v>51</v>
       </c>
-      <c r="C6" s="25" t="s">
+      <c r="C6" s="20" t="s">
         <v>233</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="D6" s="12" t="s">
         <v>234</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="E6" s="12" t="s">
         <v>235</v>
       </c>
-      <c r="F6" s="40" t="s">
+      <c r="F6" s="35" t="s">
         <v>85</v>
       </c>
-      <c r="G6" s="25" t="s">
-        <v>90</v>
-      </c>
-      <c r="H6" s="25" t="s">
-        <v>86</v>
-      </c>
-      <c r="I6" s="7"/>
+      <c r="G6" s="20" t="s">
+        <v>90</v>
+      </c>
+      <c r="H6" s="20" t="s">
+        <v>86</v>
+      </c>
+      <c r="I6" s="12"/>
     </row>
     <row r="7" spans="1:9" ht="51" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="25">
+      <c r="A7" s="20">
         <v>3</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B7" s="12" t="s">
         <v>51</v>
       </c>
-      <c r="C7" s="25" t="s">
+      <c r="C7" s="20" t="s">
         <v>236</v>
       </c>
-      <c r="D7" s="7" t="s">
+      <c r="D7" s="12" t="s">
         <v>237</v>
       </c>
-      <c r="E7" s="7" t="s">
+      <c r="E7" s="12" t="s">
         <v>238</v>
       </c>
-      <c r="F7" s="40" t="s">
+      <c r="F7" s="35" t="s">
         <v>85</v>
       </c>
-      <c r="G7" s="25" t="s">
-        <v>90</v>
-      </c>
-      <c r="H7" s="25" t="s">
-        <v>86</v>
-      </c>
-      <c r="I7" s="7"/>
+      <c r="G7" s="20" t="s">
+        <v>90</v>
+      </c>
+      <c r="H7" s="20" t="s">
+        <v>86</v>
+      </c>
+      <c r="I7" s="12"/>
     </row>
     <row r="8" spans="1:9" ht="51" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="25">
+      <c r="A8" s="20">
         <v>4</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="12" t="s">
         <v>51</v>
       </c>
-      <c r="C8" s="25" t="s">
+      <c r="C8" s="20" t="s">
         <v>239</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="D8" s="12" t="s">
         <v>240</v>
       </c>
-      <c r="E8" s="7" t="s">
+      <c r="E8" s="12" t="s">
         <v>241</v>
       </c>
-      <c r="F8" s="31" t="s">
-        <v>90</v>
-      </c>
-      <c r="G8" s="25" t="s">
+      <c r="F8" s="26" t="s">
+        <v>90</v>
+      </c>
+      <c r="G8" s="20" t="s">
         <v>97</v>
       </c>
-      <c r="H8" s="25" t="s">
-        <v>86</v>
-      </c>
-      <c r="I8" s="7"/>
+      <c r="H8" s="20" t="s">
+        <v>86</v>
+      </c>
+      <c r="I8" s="12"/>
     </row>
     <row r="9" spans="1:9" ht="51" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="26">
+      <c r="A9" s="21">
         <v>5</v>
       </c>
-      <c r="B9" s="23" t="s">
+      <c r="B9" s="18" t="s">
         <v>51</v>
       </c>
-      <c r="C9" s="26" t="s">
+      <c r="C9" s="21" t="s">
         <v>242</v>
       </c>
-      <c r="D9" s="23" t="s">
+      <c r="D9" s="18" t="s">
         <v>243</v>
       </c>
-      <c r="E9" s="23" t="s">
+      <c r="E9" s="18" t="s">
         <v>244</v>
       </c>
-      <c r="F9" s="41" t="s">
+      <c r="F9" s="36" t="s">
         <v>85</v>
       </c>
-      <c r="G9" s="26" t="s">
+      <c r="G9" s="21" t="s">
         <v>97</v>
       </c>
-      <c r="H9" s="26" t="s">
-        <v>86</v>
-      </c>
-      <c r="I9" s="23"/>
+      <c r="H9" s="21" t="s">
+        <v>86</v>
+      </c>
+      <c r="I9" s="18"/>
     </row>
     <row r="10" spans="1:9" ht="51" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="27">
+      <c r="A10" s="22">
         <v>6</v>
       </c>
-      <c r="B10" s="24" t="s">
+      <c r="B10" s="19" t="s">
         <v>245</v>
       </c>
-      <c r="C10" s="27" t="s">
+      <c r="C10" s="22" t="s">
         <v>246</v>
       </c>
-      <c r="D10" s="24" t="s">
+      <c r="D10" s="19" t="s">
         <v>247</v>
       </c>
-      <c r="E10" s="24" t="s">
+      <c r="E10" s="19" t="s">
         <v>248</v>
       </c>
-      <c r="F10" s="33" t="s">
+      <c r="F10" s="28" t="s">
         <v>85</v>
       </c>
-      <c r="G10" s="27" t="s">
+      <c r="G10" s="22" t="s">
         <v>85</v>
       </c>
-      <c r="H10" s="27" t="s">
-        <v>86</v>
-      </c>
-      <c r="I10" s="24"/>
+      <c r="H10" s="22" t="s">
+        <v>86</v>
+      </c>
+      <c r="I10" s="19"/>
     </row>
     <row r="11" spans="1:9" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="28">
+      <c r="A11" s="23">
         <v>7</v>
       </c>
-      <c r="B11" s="22" t="s">
+      <c r="B11" s="17" t="s">
         <v>245</v>
       </c>
-      <c r="C11" s="28" t="s">
+      <c r="C11" s="23" t="s">
         <v>249</v>
       </c>
-      <c r="D11" s="22" t="s">
+      <c r="D11" s="17" t="s">
         <v>250</v>
       </c>
-      <c r="E11" s="22" t="s">
+      <c r="E11" s="17" t="s">
         <v>251</v>
       </c>
-      <c r="F11" s="39" t="s">
+      <c r="F11" s="34" t="s">
         <v>85</v>
       </c>
-      <c r="G11" s="28" t="s">
+      <c r="G11" s="23" t="s">
         <v>85</v>
       </c>
-      <c r="H11" s="28" t="s">
-        <v>86</v>
-      </c>
-      <c r="I11" s="22"/>
+      <c r="H11" s="23" t="s">
+        <v>86</v>
+      </c>
+      <c r="I11" s="17"/>
     </row>
     <row r="12" spans="1:9" ht="51" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="25">
+      <c r="A12" s="20">
         <v>8</v>
       </c>
-      <c r="B12" s="7" t="s">
+      <c r="B12" s="12" t="s">
         <v>245</v>
       </c>
-      <c r="C12" s="25" t="s">
+      <c r="C12" s="20" t="s">
         <v>252</v>
       </c>
-      <c r="D12" s="7" t="s">
+      <c r="D12" s="12" t="s">
         <v>253</v>
       </c>
-      <c r="E12" s="7" t="s">
+      <c r="E12" s="12" t="s">
         <v>254</v>
       </c>
-      <c r="F12" s="31" t="s">
-        <v>90</v>
-      </c>
-      <c r="G12" s="25" t="s">
+      <c r="F12" s="26" t="s">
+        <v>90</v>
+      </c>
+      <c r="G12" s="20" t="s">
         <v>85</v>
       </c>
-      <c r="H12" s="25" t="s">
-        <v>86</v>
-      </c>
-      <c r="I12" s="7"/>
+      <c r="H12" s="20" t="s">
+        <v>86</v>
+      </c>
+      <c r="I12" s="12"/>
     </row>
     <row r="13" spans="1:9" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="25">
+      <c r="A13" s="20">
         <v>9</v>
       </c>
-      <c r="B13" s="7" t="s">
+      <c r="B13" s="12" t="s">
         <v>245</v>
       </c>
-      <c r="C13" s="25" t="s">
+      <c r="C13" s="20" t="s">
         <v>255</v>
       </c>
-      <c r="D13" s="7" t="s">
+      <c r="D13" s="12" t="s">
         <v>256</v>
       </c>
-      <c r="E13" s="7" t="s">
+      <c r="E13" s="12" t="s">
         <v>257</v>
       </c>
-      <c r="F13" s="31" t="s">
-        <v>90</v>
-      </c>
-      <c r="G13" s="25" t="s">
+      <c r="F13" s="26" t="s">
+        <v>90</v>
+      </c>
+      <c r="G13" s="20" t="s">
         <v>85</v>
       </c>
-      <c r="H13" s="25" t="s">
-        <v>86</v>
-      </c>
-      <c r="I13" s="7"/>
+      <c r="H13" s="20" t="s">
+        <v>86</v>
+      </c>
+      <c r="I13" s="12"/>
     </row>
     <row r="14" spans="1:9" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="25">
+      <c r="A14" s="20">
         <v>10</v>
       </c>
-      <c r="B14" s="7" t="s">
+      <c r="B14" s="12" t="s">
         <v>245</v>
       </c>
-      <c r="C14" s="25" t="s">
+      <c r="C14" s="20" t="s">
         <v>258</v>
       </c>
-      <c r="D14" s="7" t="s">
+      <c r="D14" s="12" t="s">
         <v>259</v>
       </c>
-      <c r="E14" s="7" t="s">
+      <c r="E14" s="12" t="s">
         <v>260</v>
       </c>
-      <c r="F14" s="40" t="s">
+      <c r="F14" s="35" t="s">
         <v>85</v>
       </c>
-      <c r="G14" s="25" t="s">
-        <v>90</v>
-      </c>
-      <c r="H14" s="25" t="s">
-        <v>86</v>
-      </c>
-      <c r="I14" s="7"/>
+      <c r="G14" s="20" t="s">
+        <v>90</v>
+      </c>
+      <c r="H14" s="20" t="s">
+        <v>86</v>
+      </c>
+      <c r="I14" s="12"/>
     </row>
     <row r="15" spans="1:9" ht="51" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="25">
+      <c r="A15" s="20">
         <v>11</v>
       </c>
-      <c r="B15" s="7" t="s">
+      <c r="B15" s="12" t="s">
         <v>245</v>
       </c>
-      <c r="C15" s="25" t="s">
+      <c r="C15" s="20" t="s">
         <v>261</v>
       </c>
-      <c r="D15" s="7" t="s">
+      <c r="D15" s="12" t="s">
         <v>262</v>
       </c>
-      <c r="E15" s="7" t="s">
+      <c r="E15" s="12" t="s">
         <v>263</v>
       </c>
-      <c r="F15" s="31" t="s">
-        <v>90</v>
-      </c>
-      <c r="G15" s="25" t="s">
-        <v>90</v>
-      </c>
-      <c r="H15" s="25" t="s">
-        <v>86</v>
-      </c>
-      <c r="I15" s="7"/>
+      <c r="F15" s="26" t="s">
+        <v>90</v>
+      </c>
+      <c r="G15" s="20" t="s">
+        <v>90</v>
+      </c>
+      <c r="H15" s="20" t="s">
+        <v>86</v>
+      </c>
+      <c r="I15" s="12"/>
     </row>
     <row r="16" spans="1:9" ht="36" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="26">
+      <c r="A16" s="21">
         <v>12</v>
       </c>
-      <c r="B16" s="23" t="s">
+      <c r="B16" s="18" t="s">
         <v>245</v>
       </c>
-      <c r="C16" s="26" t="s">
+      <c r="C16" s="21" t="s">
         <v>264</v>
       </c>
-      <c r="D16" s="23" t="s">
+      <c r="D16" s="18" t="s">
         <v>265</v>
       </c>
-      <c r="E16" s="23" t="s">
+      <c r="E16" s="18" t="s">
         <v>266</v>
       </c>
-      <c r="F16" s="32" t="s">
-        <v>90</v>
-      </c>
-      <c r="G16" s="26" t="s">
-        <v>90</v>
-      </c>
-      <c r="H16" s="26" t="s">
-        <v>86</v>
-      </c>
-      <c r="I16" s="23"/>
+      <c r="F16" s="27" t="s">
+        <v>90</v>
+      </c>
+      <c r="G16" s="21" t="s">
+        <v>90</v>
+      </c>
+      <c r="H16" s="21" t="s">
+        <v>86</v>
+      </c>
+      <c r="I16" s="18"/>
     </row>
     <row r="17" spans="1:9" ht="96" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="27">
+      <c r="A17" s="22">
         <v>13</v>
       </c>
-      <c r="B17" s="24" t="s">
+      <c r="B17" s="19" t="s">
         <v>267</v>
       </c>
-      <c r="C17" s="27" t="s">
+      <c r="C17" s="22" t="s">
         <v>268</v>
       </c>
-      <c r="D17" s="24" t="s">
+      <c r="D17" s="19" t="s">
         <v>269</v>
       </c>
-      <c r="E17" s="24" t="s">
+      <c r="E17" s="19" t="s">
         <v>270</v>
       </c>
-      <c r="F17" s="38" t="s">
+      <c r="F17" s="33" t="s">
         <v>84</v>
       </c>
-      <c r="G17" s="27" t="s">
+      <c r="G17" s="22" t="s">
         <v>85</v>
       </c>
-      <c r="H17" s="27" t="s">
-        <v>86</v>
-      </c>
-      <c r="I17" s="24"/>
+      <c r="H17" s="22" t="s">
+        <v>86</v>
+      </c>
+      <c r="I17" s="19"/>
     </row>
     <row r="18" spans="1:9" ht="81" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="28">
+      <c r="A18" s="23">
         <v>14</v>
       </c>
-      <c r="B18" s="22" t="s">
+      <c r="B18" s="17" t="s">
         <v>267</v>
       </c>
-      <c r="C18" s="28" t="s">
+      <c r="C18" s="23" t="s">
         <v>271</v>
       </c>
-      <c r="D18" s="22" t="s">
+      <c r="D18" s="17" t="s">
         <v>272</v>
       </c>
-      <c r="E18" s="22" t="s">
+      <c r="E18" s="17" t="s">
         <v>273</v>
       </c>
-      <c r="F18" s="39" t="s">
+      <c r="F18" s="34" t="s">
         <v>85</v>
       </c>
-      <c r="G18" s="28" t="s">
-        <v>90</v>
-      </c>
-      <c r="H18" s="28" t="s">
-        <v>86</v>
-      </c>
-      <c r="I18" s="22"/>
+      <c r="G18" s="23" t="s">
+        <v>90</v>
+      </c>
+      <c r="H18" s="23" t="s">
+        <v>86</v>
+      </c>
+      <c r="I18" s="17"/>
     </row>
     <row r="19" spans="1:9" ht="66" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="25">
+      <c r="A19" s="20">
         <v>15</v>
       </c>
-      <c r="B19" s="7" t="s">
+      <c r="B19" s="12" t="s">
         <v>267</v>
       </c>
-      <c r="C19" s="25" t="s">
+      <c r="C19" s="20" t="s">
         <v>274</v>
       </c>
-      <c r="D19" s="7" t="s">
+      <c r="D19" s="12" t="s">
         <v>275</v>
       </c>
-      <c r="E19" s="7" t="s">
+      <c r="E19" s="12" t="s">
         <v>276</v>
       </c>
-      <c r="F19" s="31" t="s">
-        <v>90</v>
-      </c>
-      <c r="G19" s="25" t="s">
-        <v>90</v>
-      </c>
-      <c r="H19" s="25" t="s">
-        <v>86</v>
-      </c>
-      <c r="I19" s="7"/>
+      <c r="F19" s="26" t="s">
+        <v>90</v>
+      </c>
+      <c r="G19" s="20" t="s">
+        <v>90</v>
+      </c>
+      <c r="H19" s="20" t="s">
+        <v>86</v>
+      </c>
+      <c r="I19" s="12"/>
     </row>
     <row r="20" spans="1:9" ht="66" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="25">
+      <c r="A20" s="20">
         <v>16</v>
       </c>
-      <c r="B20" s="7" t="s">
+      <c r="B20" s="12" t="s">
         <v>267</v>
       </c>
-      <c r="C20" s="25" t="s">
+      <c r="C20" s="20" t="s">
         <v>277</v>
       </c>
-      <c r="D20" s="7" t="s">
+      <c r="D20" s="12" t="s">
         <v>278</v>
       </c>
-      <c r="E20" s="7" t="s">
+      <c r="E20" s="12" t="s">
         <v>279</v>
       </c>
-      <c r="F20" s="31" t="s">
-        <v>90</v>
-      </c>
-      <c r="G20" s="25" t="s">
-        <v>90</v>
-      </c>
-      <c r="H20" s="25" t="s">
-        <v>86</v>
-      </c>
-      <c r="I20" s="7"/>
+      <c r="F20" s="26" t="s">
+        <v>90</v>
+      </c>
+      <c r="G20" s="20" t="s">
+        <v>90</v>
+      </c>
+      <c r="H20" s="20" t="s">
+        <v>86</v>
+      </c>
+      <c r="I20" s="12"/>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
@@ -4328,7 +4451,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:I20"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.7109375" customWidth="1"/>
     <col min="2" max="2" width="24.7109375" customWidth="1"/>
@@ -4346,424 +4469,424 @@
       </c>
     </row>
     <row r="2" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="20" t="s">
+      <c r="A2" s="39" t="s">
         <v>281</v>
       </c>
-      <c r="B2" s="20"/>
-      <c r="C2" s="20"/>
-      <c r="D2" s="20"/>
-      <c r="E2" s="20"/>
-      <c r="F2" s="20"/>
-      <c r="G2" s="20"/>
-      <c r="H2" s="20"/>
-      <c r="I2" s="20"/>
+      <c r="B2" s="39"/>
+      <c r="C2" s="39"/>
+      <c r="D2" s="39"/>
+      <c r="E2" s="39"/>
+      <c r="F2" s="39"/>
+      <c r="G2" s="39"/>
+      <c r="H2" s="39"/>
+      <c r="I2" s="39"/>
     </row>
     <row r="4" spans="1:9" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="11" t="s">
         <v>71</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="11" t="s">
         <v>73</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="11" t="s">
         <v>74</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="11" t="s">
         <v>75</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="F4" s="11" t="s">
         <v>76</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="G4" s="11" t="s">
         <v>77</v>
       </c>
-      <c r="H4" s="3" t="s">
+      <c r="H4" s="11" t="s">
         <v>78</v>
       </c>
-      <c r="I4" s="3" t="s">
+      <c r="I4" s="11" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="25">
+      <c r="A5" s="20">
         <v>1</v>
       </c>
-      <c r="B5" s="7" t="s">
+      <c r="B5" s="12" t="s">
         <v>282</v>
       </c>
-      <c r="C5" s="25" t="s">
+      <c r="C5" s="20" t="s">
         <v>283</v>
       </c>
-      <c r="D5" s="7" t="s">
+      <c r="D5" s="12" t="s">
         <v>284</v>
       </c>
-      <c r="E5" s="7" t="s">
+      <c r="E5" s="12" t="s">
         <v>285</v>
       </c>
-      <c r="F5" s="40" t="s">
+      <c r="F5" s="35" t="s">
         <v>85</v>
       </c>
-      <c r="G5" s="25" t="s">
-        <v>90</v>
-      </c>
-      <c r="H5" s="25" t="s">
-        <v>86</v>
-      </c>
-      <c r="I5" s="7"/>
+      <c r="G5" s="20" t="s">
+        <v>90</v>
+      </c>
+      <c r="H5" s="20" t="s">
+        <v>86</v>
+      </c>
+      <c r="I5" s="12"/>
     </row>
     <row r="6" spans="1:9" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="25">
+      <c r="A6" s="20">
         <v>2</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="B6" s="12" t="s">
         <v>282</v>
       </c>
-      <c r="C6" s="25" t="s">
+      <c r="C6" s="20" t="s">
         <v>286</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="D6" s="12" t="s">
         <v>287</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="E6" s="12" t="s">
         <v>288</v>
       </c>
-      <c r="F6" s="40" t="s">
+      <c r="F6" s="35" t="s">
         <v>85</v>
       </c>
-      <c r="G6" s="25" t="s">
-        <v>90</v>
-      </c>
-      <c r="H6" s="25" t="s">
-        <v>86</v>
-      </c>
-      <c r="I6" s="7"/>
+      <c r="G6" s="20" t="s">
+        <v>90</v>
+      </c>
+      <c r="H6" s="20" t="s">
+        <v>86</v>
+      </c>
+      <c r="I6" s="12"/>
     </row>
     <row r="7" spans="1:9" ht="51" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="25">
+      <c r="A7" s="20">
         <v>3</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B7" s="12" t="s">
         <v>282</v>
       </c>
-      <c r="C7" s="25" t="s">
+      <c r="C7" s="20" t="s">
         <v>289</v>
       </c>
-      <c r="D7" s="7" t="s">
+      <c r="D7" s="12" t="s">
         <v>290</v>
       </c>
-      <c r="E7" s="7" t="s">
+      <c r="E7" s="12" t="s">
         <v>291</v>
       </c>
-      <c r="F7" s="40" t="s">
+      <c r="F7" s="35" t="s">
         <v>85</v>
       </c>
-      <c r="G7" s="25" t="s">
+      <c r="G7" s="20" t="s">
         <v>85</v>
       </c>
-      <c r="H7" s="25" t="s">
-        <v>86</v>
-      </c>
-      <c r="I7" s="7"/>
+      <c r="H7" s="20" t="s">
+        <v>86</v>
+      </c>
+      <c r="I7" s="12"/>
     </row>
     <row r="8" spans="1:9" ht="51" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="25">
+      <c r="A8" s="20">
         <v>4</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="12" t="s">
         <v>282</v>
       </c>
-      <c r="C8" s="25" t="s">
+      <c r="C8" s="20" t="s">
         <v>292</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="D8" s="12" t="s">
         <v>293</v>
       </c>
-      <c r="E8" s="7" t="s">
+      <c r="E8" s="12" t="s">
         <v>294</v>
       </c>
-      <c r="F8" s="31" t="s">
-        <v>90</v>
-      </c>
-      <c r="G8" s="25" t="s">
-        <v>90</v>
-      </c>
-      <c r="H8" s="25" t="s">
-        <v>86</v>
-      </c>
-      <c r="I8" s="7"/>
+      <c r="F8" s="26" t="s">
+        <v>90</v>
+      </c>
+      <c r="G8" s="20" t="s">
+        <v>90</v>
+      </c>
+      <c r="H8" s="20" t="s">
+        <v>86</v>
+      </c>
+      <c r="I8" s="12"/>
     </row>
     <row r="9" spans="1:9" ht="51" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="25">
+      <c r="A9" s="20">
         <v>5</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="12" t="s">
         <v>282</v>
       </c>
-      <c r="C9" s="25" t="s">
+      <c r="C9" s="20" t="s">
         <v>295</v>
       </c>
-      <c r="D9" s="7" t="s">
+      <c r="D9" s="12" t="s">
         <v>296</v>
       </c>
-      <c r="E9" s="7" t="s">
+      <c r="E9" s="12" t="s">
         <v>297</v>
       </c>
-      <c r="F9" s="31" t="s">
-        <v>90</v>
-      </c>
-      <c r="G9" s="25" t="s">
-        <v>90</v>
-      </c>
-      <c r="H9" s="25" t="s">
-        <v>86</v>
-      </c>
-      <c r="I9" s="7"/>
+      <c r="F9" s="26" t="s">
+        <v>90</v>
+      </c>
+      <c r="G9" s="20" t="s">
+        <v>90</v>
+      </c>
+      <c r="H9" s="20" t="s">
+        <v>86</v>
+      </c>
+      <c r="I9" s="12"/>
     </row>
     <row r="10" spans="1:9" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="25">
+      <c r="A10" s="20">
         <v>6</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="B10" s="12" t="s">
         <v>282</v>
       </c>
-      <c r="C10" s="25" t="s">
+      <c r="C10" s="20" t="s">
         <v>298</v>
       </c>
-      <c r="D10" s="7" t="s">
+      <c r="D10" s="12" t="s">
         <v>299</v>
       </c>
-      <c r="E10" s="7" t="s">
+      <c r="E10" s="12" t="s">
         <v>300</v>
       </c>
-      <c r="F10" s="31" t="s">
-        <v>90</v>
-      </c>
-      <c r="G10" s="25" t="s">
-        <v>90</v>
-      </c>
-      <c r="H10" s="25" t="s">
-        <v>86</v>
-      </c>
-      <c r="I10" s="7"/>
+      <c r="F10" s="26" t="s">
+        <v>90</v>
+      </c>
+      <c r="G10" s="20" t="s">
+        <v>90</v>
+      </c>
+      <c r="H10" s="20" t="s">
+        <v>86</v>
+      </c>
+      <c r="I10" s="12"/>
     </row>
     <row r="11" spans="1:9" ht="36" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="26">
+      <c r="A11" s="21">
         <v>7</v>
       </c>
-      <c r="B11" s="23" t="s">
+      <c r="B11" s="18" t="s">
         <v>282</v>
       </c>
-      <c r="C11" s="26" t="s">
+      <c r="C11" s="21" t="s">
         <v>301</v>
       </c>
-      <c r="D11" s="23" t="s">
+      <c r="D11" s="18" t="s">
         <v>302</v>
       </c>
-      <c r="E11" s="23" t="s">
+      <c r="E11" s="18" t="s">
         <v>303</v>
       </c>
-      <c r="F11" s="32" t="s">
-        <v>90</v>
-      </c>
-      <c r="G11" s="26" t="s">
+      <c r="F11" s="27" t="s">
+        <v>90</v>
+      </c>
+      <c r="G11" s="21" t="s">
         <v>97</v>
       </c>
-      <c r="H11" s="26" t="s">
-        <v>86</v>
-      </c>
-      <c r="I11" s="23"/>
+      <c r="H11" s="21" t="s">
+        <v>86</v>
+      </c>
+      <c r="I11" s="18"/>
     </row>
     <row r="12" spans="1:9" ht="51" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="27">
+      <c r="A12" s="22">
         <v>8</v>
       </c>
-      <c r="B12" s="24" t="s">
+      <c r="B12" s="19" t="s">
         <v>304</v>
       </c>
-      <c r="C12" s="27" t="s">
+      <c r="C12" s="22" t="s">
         <v>305</v>
       </c>
-      <c r="D12" s="24" t="s">
+      <c r="D12" s="19" t="s">
         <v>306</v>
       </c>
-      <c r="E12" s="24" t="s">
+      <c r="E12" s="19" t="s">
         <v>307</v>
       </c>
-      <c r="F12" s="36" t="s">
-        <v>90</v>
-      </c>
-      <c r="G12" s="27" t="s">
-        <v>90</v>
-      </c>
-      <c r="H12" s="27" t="s">
-        <v>86</v>
-      </c>
-      <c r="I12" s="24"/>
+      <c r="F12" s="31" t="s">
+        <v>90</v>
+      </c>
+      <c r="G12" s="22" t="s">
+        <v>90</v>
+      </c>
+      <c r="H12" s="22" t="s">
+        <v>86</v>
+      </c>
+      <c r="I12" s="19"/>
     </row>
     <row r="13" spans="1:9" ht="81" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="28">
+      <c r="A13" s="23">
         <v>9</v>
       </c>
-      <c r="B13" s="22" t="s">
+      <c r="B13" s="17" t="s">
         <v>304</v>
       </c>
-      <c r="C13" s="28" t="s">
+      <c r="C13" s="23" t="s">
         <v>308</v>
       </c>
-      <c r="D13" s="22" t="s">
+      <c r="D13" s="17" t="s">
         <v>309</v>
       </c>
-      <c r="E13" s="22" t="s">
+      <c r="E13" s="17" t="s">
         <v>310</v>
       </c>
-      <c r="F13" s="34" t="s">
-        <v>90</v>
-      </c>
-      <c r="G13" s="28" t="s">
-        <v>90</v>
-      </c>
-      <c r="H13" s="28" t="s">
-        <v>86</v>
-      </c>
-      <c r="I13" s="22"/>
+      <c r="F13" s="29" t="s">
+        <v>90</v>
+      </c>
+      <c r="G13" s="23" t="s">
+        <v>90</v>
+      </c>
+      <c r="H13" s="23" t="s">
+        <v>86</v>
+      </c>
+      <c r="I13" s="17"/>
     </row>
     <row r="14" spans="1:9" ht="51" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="26">
+      <c r="A14" s="21">
         <v>10</v>
       </c>
-      <c r="B14" s="23" t="s">
+      <c r="B14" s="18" t="s">
         <v>304</v>
       </c>
-      <c r="C14" s="26" t="s">
+      <c r="C14" s="21" t="s">
         <v>311</v>
       </c>
-      <c r="D14" s="23" t="s">
+      <c r="D14" s="18" t="s">
         <v>312</v>
       </c>
-      <c r="E14" s="23" t="s">
+      <c r="E14" s="18" t="s">
         <v>313</v>
       </c>
-      <c r="F14" s="32" t="s">
-        <v>90</v>
-      </c>
-      <c r="G14" s="26" t="s">
+      <c r="F14" s="27" t="s">
+        <v>90</v>
+      </c>
+      <c r="G14" s="21" t="s">
         <v>97</v>
       </c>
-      <c r="H14" s="26" t="s">
-        <v>86</v>
-      </c>
-      <c r="I14" s="23"/>
+      <c r="H14" s="21" t="s">
+        <v>86</v>
+      </c>
+      <c r="I14" s="18"/>
     </row>
     <row r="15" spans="1:9" ht="81" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="27">
+      <c r="A15" s="22">
         <v>11</v>
       </c>
-      <c r="B15" s="24" t="s">
+      <c r="B15" s="19" t="s">
         <v>314</v>
       </c>
-      <c r="C15" s="27" t="s">
+      <c r="C15" s="22" t="s">
         <v>315</v>
       </c>
-      <c r="D15" s="24" t="s">
+      <c r="D15" s="19" t="s">
         <v>316</v>
       </c>
-      <c r="E15" s="24" t="s">
+      <c r="E15" s="19" t="s">
         <v>317</v>
       </c>
-      <c r="F15" s="36" t="s">
-        <v>90</v>
-      </c>
-      <c r="G15" s="27" t="s">
-        <v>90</v>
-      </c>
-      <c r="H15" s="27" t="s">
-        <v>86</v>
-      </c>
-      <c r="I15" s="24"/>
+      <c r="F15" s="31" t="s">
+        <v>90</v>
+      </c>
+      <c r="G15" s="22" t="s">
+        <v>90</v>
+      </c>
+      <c r="H15" s="22" t="s">
+        <v>86</v>
+      </c>
+      <c r="I15" s="19"/>
     </row>
     <row r="16" spans="1:9" ht="51" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="29">
+      <c r="A16" s="24">
         <v>12</v>
       </c>
-      <c r="B16" s="21" t="s">
+      <c r="B16" s="16" t="s">
         <v>314</v>
       </c>
-      <c r="C16" s="29" t="s">
+      <c r="C16" s="24" t="s">
         <v>318</v>
       </c>
-      <c r="D16" s="21" t="s">
+      <c r="D16" s="16" t="s">
         <v>319</v>
       </c>
-      <c r="E16" s="21" t="s">
+      <c r="E16" s="16" t="s">
         <v>320</v>
       </c>
-      <c r="F16" s="37" t="s">
-        <v>90</v>
-      </c>
-      <c r="G16" s="29" t="s">
+      <c r="F16" s="32" t="s">
+        <v>90</v>
+      </c>
+      <c r="G16" s="24" t="s">
         <v>97</v>
       </c>
-      <c r="H16" s="29" t="s">
-        <v>86</v>
-      </c>
-      <c r="I16" s="21"/>
+      <c r="H16" s="24" t="s">
+        <v>86</v>
+      </c>
+      <c r="I16" s="16"/>
     </row>
     <row r="17" spans="1:9" ht="66" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="27">
+      <c r="A17" s="22">
         <v>13</v>
       </c>
-      <c r="B17" s="24" t="s">
+      <c r="B17" s="19" t="s">
         <v>321</v>
       </c>
-      <c r="C17" s="27" t="s">
+      <c r="C17" s="22" t="s">
         <v>322</v>
       </c>
-      <c r="D17" s="24" t="s">
+      <c r="D17" s="19" t="s">
         <v>323</v>
       </c>
-      <c r="E17" s="24" t="s">
+      <c r="E17" s="19" t="s">
         <v>324</v>
       </c>
-      <c r="F17" s="36" t="s">
-        <v>90</v>
-      </c>
-      <c r="G17" s="27" t="s">
-        <v>90</v>
-      </c>
-      <c r="H17" s="27" t="s">
-        <v>86</v>
-      </c>
-      <c r="I17" s="24"/>
+      <c r="F17" s="31" t="s">
+        <v>90</v>
+      </c>
+      <c r="G17" s="22" t="s">
+        <v>90</v>
+      </c>
+      <c r="H17" s="22" t="s">
+        <v>86</v>
+      </c>
+      <c r="I17" s="19"/>
     </row>
     <row r="18" spans="1:9" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="28">
+      <c r="A18" s="23">
         <v>14</v>
       </c>
-      <c r="B18" s="22" t="s">
+      <c r="B18" s="17" t="s">
         <v>321</v>
       </c>
-      <c r="C18" s="28" t="s">
+      <c r="C18" s="23" t="s">
         <v>325</v>
       </c>
-      <c r="D18" s="22" t="s">
+      <c r="D18" s="17" t="s">
         <v>326</v>
       </c>
-      <c r="E18" s="22" t="s">
+      <c r="E18" s="17" t="s">
         <v>327</v>
       </c>
-      <c r="F18" s="34" t="s">
-        <v>90</v>
-      </c>
-      <c r="G18" s="28" t="s">
+      <c r="F18" s="29" t="s">
+        <v>90</v>
+      </c>
+      <c r="G18" s="23" t="s">
         <v>97</v>
       </c>
-      <c r="H18" s="28" t="s">
-        <v>86</v>
-      </c>
-      <c r="I18" s="22"/>
+      <c r="H18" s="23" t="s">
+        <v>86</v>
+      </c>
+      <c r="I18" s="17"/>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
@@ -4813,7 +4936,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:I23"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.7109375" customWidth="1"/>
     <col min="2" max="2" width="24.7109375" customWidth="1"/>
@@ -4831,505 +4954,505 @@
       </c>
     </row>
     <row r="2" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="20" t="s">
+      <c r="A2" s="39" t="s">
         <v>329</v>
       </c>
-      <c r="B2" s="20"/>
-      <c r="C2" s="20"/>
-      <c r="D2" s="20"/>
-      <c r="E2" s="20"/>
-      <c r="F2" s="20"/>
-      <c r="G2" s="20"/>
-      <c r="H2" s="20"/>
-      <c r="I2" s="20"/>
+      <c r="B2" s="39"/>
+      <c r="C2" s="39"/>
+      <c r="D2" s="39"/>
+      <c r="E2" s="39"/>
+      <c r="F2" s="39"/>
+      <c r="G2" s="39"/>
+      <c r="H2" s="39"/>
+      <c r="I2" s="39"/>
     </row>
     <row r="4" spans="1:9" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="11" t="s">
         <v>71</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="11" t="s">
         <v>73</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="11" t="s">
         <v>74</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="11" t="s">
         <v>75</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="F4" s="11" t="s">
         <v>76</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="G4" s="11" t="s">
         <v>77</v>
       </c>
-      <c r="H4" s="3" t="s">
+      <c r="H4" s="11" t="s">
         <v>78</v>
       </c>
-      <c r="I4" s="3" t="s">
+      <c r="I4" s="11" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="25">
+      <c r="A5" s="20">
         <v>1</v>
       </c>
-      <c r="B5" s="7" t="s">
+      <c r="B5" s="12" t="s">
         <v>330</v>
       </c>
-      <c r="C5" s="25" t="s">
+      <c r="C5" s="20" t="s">
         <v>331</v>
       </c>
-      <c r="D5" s="7" t="s">
+      <c r="D5" s="12" t="s">
         <v>332</v>
       </c>
-      <c r="E5" s="7" t="s">
+      <c r="E5" s="12" t="s">
         <v>333</v>
       </c>
-      <c r="F5" s="31" t="s">
-        <v>90</v>
-      </c>
-      <c r="G5" s="25" t="s">
-        <v>90</v>
-      </c>
-      <c r="H5" s="25" t="s">
-        <v>86</v>
-      </c>
-      <c r="I5" s="7"/>
+      <c r="F5" s="26" t="s">
+        <v>90</v>
+      </c>
+      <c r="G5" s="20" t="s">
+        <v>90</v>
+      </c>
+      <c r="H5" s="20" t="s">
+        <v>86</v>
+      </c>
+      <c r="I5" s="12"/>
     </row>
     <row r="6" spans="1:9" ht="51" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="25">
+      <c r="A6" s="20">
         <v>2</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="B6" s="12" t="s">
         <v>330</v>
       </c>
-      <c r="C6" s="25" t="s">
+      <c r="C6" s="20" t="s">
         <v>334</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="D6" s="12" t="s">
         <v>335</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="E6" s="12" t="s">
         <v>336</v>
       </c>
-      <c r="F6" s="31" t="s">
-        <v>90</v>
-      </c>
-      <c r="G6" s="25" t="s">
-        <v>90</v>
-      </c>
-      <c r="H6" s="25" t="s">
-        <v>86</v>
-      </c>
-      <c r="I6" s="7"/>
+      <c r="F6" s="26" t="s">
+        <v>90</v>
+      </c>
+      <c r="G6" s="20" t="s">
+        <v>90</v>
+      </c>
+      <c r="H6" s="20" t="s">
+        <v>86</v>
+      </c>
+      <c r="I6" s="12"/>
     </row>
     <row r="7" spans="1:9" ht="51" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="26">
+      <c r="A7" s="21">
         <v>3</v>
       </c>
-      <c r="B7" s="23" t="s">
+      <c r="B7" s="18" t="s">
         <v>330</v>
       </c>
-      <c r="C7" s="26" t="s">
+      <c r="C7" s="21" t="s">
         <v>337</v>
       </c>
-      <c r="D7" s="23" t="s">
+      <c r="D7" s="18" t="s">
         <v>338</v>
       </c>
-      <c r="E7" s="23" t="s">
+      <c r="E7" s="18" t="s">
         <v>339</v>
       </c>
-      <c r="F7" s="32" t="s">
-        <v>90</v>
-      </c>
-      <c r="G7" s="26" t="s">
+      <c r="F7" s="27" t="s">
+        <v>90</v>
+      </c>
+      <c r="G7" s="21" t="s">
         <v>97</v>
       </c>
-      <c r="H7" s="26" t="s">
-        <v>86</v>
-      </c>
-      <c r="I7" s="23"/>
+      <c r="H7" s="21" t="s">
+        <v>86</v>
+      </c>
+      <c r="I7" s="18"/>
     </row>
     <row r="8" spans="1:9" ht="66" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="27">
+      <c r="A8" s="22">
         <v>4</v>
       </c>
-      <c r="B8" s="24" t="s">
+      <c r="B8" s="19" t="s">
         <v>340</v>
       </c>
-      <c r="C8" s="27" t="s">
+      <c r="C8" s="22" t="s">
         <v>341</v>
       </c>
-      <c r="D8" s="24" t="s">
+      <c r="D8" s="19" t="s">
         <v>342</v>
       </c>
-      <c r="E8" s="24" t="s">
+      <c r="E8" s="19" t="s">
         <v>343</v>
       </c>
-      <c r="F8" s="36" t="s">
-        <v>90</v>
-      </c>
-      <c r="G8" s="27" t="s">
-        <v>90</v>
-      </c>
-      <c r="H8" s="27" t="s">
-        <v>86</v>
-      </c>
-      <c r="I8" s="24"/>
+      <c r="F8" s="31" t="s">
+        <v>90</v>
+      </c>
+      <c r="G8" s="22" t="s">
+        <v>90</v>
+      </c>
+      <c r="H8" s="22" t="s">
+        <v>86</v>
+      </c>
+      <c r="I8" s="19"/>
     </row>
     <row r="9" spans="1:9" ht="51" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="28">
+      <c r="A9" s="23">
         <v>5</v>
       </c>
-      <c r="B9" s="22" t="s">
+      <c r="B9" s="17" t="s">
         <v>340</v>
       </c>
-      <c r="C9" s="28" t="s">
+      <c r="C9" s="23" t="s">
         <v>344</v>
       </c>
-      <c r="D9" s="22" t="s">
+      <c r="D9" s="17" t="s">
         <v>345</v>
       </c>
-      <c r="E9" s="22" t="s">
+      <c r="E9" s="17" t="s">
         <v>346</v>
       </c>
-      <c r="F9" s="34" t="s">
-        <v>90</v>
-      </c>
-      <c r="G9" s="28" t="s">
+      <c r="F9" s="29" t="s">
+        <v>90</v>
+      </c>
+      <c r="G9" s="23" t="s">
         <v>97</v>
       </c>
-      <c r="H9" s="28" t="s">
-        <v>86</v>
-      </c>
-      <c r="I9" s="22"/>
+      <c r="H9" s="23" t="s">
+        <v>86</v>
+      </c>
+      <c r="I9" s="17"/>
     </row>
     <row r="10" spans="1:9" ht="51" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="26">
+      <c r="A10" s="21">
         <v>6</v>
       </c>
-      <c r="B10" s="23" t="s">
+      <c r="B10" s="18" t="s">
         <v>340</v>
       </c>
-      <c r="C10" s="26" t="s">
+      <c r="C10" s="21" t="s">
         <v>347</v>
       </c>
-      <c r="D10" s="23" t="s">
+      <c r="D10" s="18" t="s">
         <v>348</v>
       </c>
-      <c r="E10" s="23" t="s">
+      <c r="E10" s="18" t="s">
         <v>279</v>
       </c>
-      <c r="F10" s="32" t="s">
-        <v>90</v>
-      </c>
-      <c r="G10" s="26" t="s">
+      <c r="F10" s="27" t="s">
+        <v>90</v>
+      </c>
+      <c r="G10" s="21" t="s">
         <v>97</v>
       </c>
-      <c r="H10" s="26" t="s">
-        <v>86</v>
-      </c>
-      <c r="I10" s="23"/>
+      <c r="H10" s="21" t="s">
+        <v>86</v>
+      </c>
+      <c r="I10" s="18"/>
     </row>
     <row r="11" spans="1:9" ht="66" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="27">
+      <c r="A11" s="22">
         <v>7</v>
       </c>
-      <c r="B11" s="24" t="s">
+      <c r="B11" s="19" t="s">
         <v>349</v>
       </c>
-      <c r="C11" s="27" t="s">
+      <c r="C11" s="22" t="s">
         <v>350</v>
       </c>
-      <c r="D11" s="24" t="s">
+      <c r="D11" s="19" t="s">
         <v>351</v>
       </c>
-      <c r="E11" s="24" t="s">
+      <c r="E11" s="19" t="s">
         <v>352</v>
       </c>
-      <c r="F11" s="33" t="s">
+      <c r="F11" s="28" t="s">
         <v>85</v>
       </c>
-      <c r="G11" s="27" t="s">
+      <c r="G11" s="22" t="s">
         <v>85</v>
       </c>
-      <c r="H11" s="27" t="s">
-        <v>86</v>
-      </c>
-      <c r="I11" s="24"/>
+      <c r="H11" s="22" t="s">
+        <v>86</v>
+      </c>
+      <c r="I11" s="19"/>
     </row>
     <row r="12" spans="1:9" ht="51" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="28">
+      <c r="A12" s="23">
         <v>8</v>
       </c>
-      <c r="B12" s="22" t="s">
+      <c r="B12" s="17" t="s">
         <v>349</v>
       </c>
-      <c r="C12" s="28" t="s">
+      <c r="C12" s="23" t="s">
         <v>353</v>
       </c>
-      <c r="D12" s="22" t="s">
+      <c r="D12" s="17" t="s">
         <v>354</v>
       </c>
-      <c r="E12" s="22" t="s">
+      <c r="E12" s="17" t="s">
         <v>355</v>
       </c>
-      <c r="F12" s="34" t="s">
-        <v>90</v>
-      </c>
-      <c r="G12" s="28" t="s">
-        <v>90</v>
-      </c>
-      <c r="H12" s="28" t="s">
-        <v>86</v>
-      </c>
-      <c r="I12" s="22"/>
+      <c r="F12" s="29" t="s">
+        <v>90</v>
+      </c>
+      <c r="G12" s="23" t="s">
+        <v>90</v>
+      </c>
+      <c r="H12" s="23" t="s">
+        <v>86</v>
+      </c>
+      <c r="I12" s="17"/>
     </row>
     <row r="13" spans="1:9" ht="81" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="25">
+      <c r="A13" s="20">
         <v>9</v>
       </c>
-      <c r="B13" s="7" t="s">
+      <c r="B13" s="12" t="s">
         <v>349</v>
       </c>
-      <c r="C13" s="25" t="s">
+      <c r="C13" s="20" t="s">
         <v>356</v>
       </c>
-      <c r="D13" s="7" t="s">
+      <c r="D13" s="12" t="s">
         <v>357</v>
       </c>
-      <c r="E13" s="7" t="s">
+      <c r="E13" s="12" t="s">
         <v>358</v>
       </c>
-      <c r="F13" s="31" t="s">
-        <v>90</v>
-      </c>
-      <c r="G13" s="25" t="s">
-        <v>90</v>
-      </c>
-      <c r="H13" s="25" t="s">
-        <v>86</v>
-      </c>
-      <c r="I13" s="7"/>
+      <c r="F13" s="26" t="s">
+        <v>90</v>
+      </c>
+      <c r="G13" s="20" t="s">
+        <v>90</v>
+      </c>
+      <c r="H13" s="20" t="s">
+        <v>86</v>
+      </c>
+      <c r="I13" s="12"/>
     </row>
     <row r="14" spans="1:9" ht="51" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="25">
+      <c r="A14" s="20">
         <v>10</v>
       </c>
-      <c r="B14" s="7" t="s">
+      <c r="B14" s="12" t="s">
         <v>349</v>
       </c>
-      <c r="C14" s="25" t="s">
+      <c r="C14" s="20" t="s">
         <v>359</v>
       </c>
-      <c r="D14" s="7" t="s">
+      <c r="D14" s="12" t="s">
         <v>360</v>
       </c>
-      <c r="E14" s="7" t="s">
+      <c r="E14" s="12" t="s">
         <v>361</v>
       </c>
-      <c r="F14" s="31" t="s">
-        <v>90</v>
-      </c>
-      <c r="G14" s="25" t="s">
-        <v>90</v>
-      </c>
-      <c r="H14" s="25" t="s">
-        <v>86</v>
-      </c>
-      <c r="I14" s="7"/>
+      <c r="F14" s="26" t="s">
+        <v>90</v>
+      </c>
+      <c r="G14" s="20" t="s">
+        <v>90</v>
+      </c>
+      <c r="H14" s="20" t="s">
+        <v>86</v>
+      </c>
+      <c r="I14" s="12"/>
     </row>
     <row r="15" spans="1:9" ht="66" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="25">
+      <c r="A15" s="20">
         <v>11</v>
       </c>
-      <c r="B15" s="7" t="s">
+      <c r="B15" s="12" t="s">
         <v>349</v>
       </c>
-      <c r="C15" s="25" t="s">
+      <c r="C15" s="20" t="s">
         <v>362</v>
       </c>
-      <c r="D15" s="7" t="s">
+      <c r="D15" s="12" t="s">
         <v>363</v>
       </c>
-      <c r="E15" s="7" t="s">
+      <c r="E15" s="12" t="s">
         <v>364</v>
       </c>
-      <c r="F15" s="31" t="s">
-        <v>90</v>
-      </c>
-      <c r="G15" s="25" t="s">
+      <c r="F15" s="26" t="s">
+        <v>90</v>
+      </c>
+      <c r="G15" s="20" t="s">
         <v>97</v>
       </c>
-      <c r="H15" s="25" t="s">
-        <v>86</v>
-      </c>
-      <c r="I15" s="7"/>
+      <c r="H15" s="20" t="s">
+        <v>86</v>
+      </c>
+      <c r="I15" s="12"/>
     </row>
     <row r="16" spans="1:9" ht="51" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="25">
+      <c r="A16" s="20">
         <v>12</v>
       </c>
-      <c r="B16" s="7" t="s">
+      <c r="B16" s="12" t="s">
         <v>349</v>
       </c>
-      <c r="C16" s="25" t="s">
+      <c r="C16" s="20" t="s">
         <v>365</v>
       </c>
-      <c r="D16" s="7" t="s">
+      <c r="D16" s="12" t="s">
         <v>366</v>
       </c>
-      <c r="E16" s="7" t="s">
+      <c r="E16" s="12" t="s">
         <v>367</v>
       </c>
-      <c r="F16" s="31" t="s">
-        <v>90</v>
-      </c>
-      <c r="G16" s="25" t="s">
+      <c r="F16" s="26" t="s">
+        <v>90</v>
+      </c>
+      <c r="G16" s="20" t="s">
         <v>97</v>
       </c>
-      <c r="H16" s="25" t="s">
-        <v>86</v>
-      </c>
-      <c r="I16" s="7"/>
+      <c r="H16" s="20" t="s">
+        <v>86</v>
+      </c>
+      <c r="I16" s="12"/>
     </row>
     <row r="17" spans="1:9" ht="36" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="26">
+      <c r="A17" s="21">
         <v>13</v>
       </c>
-      <c r="B17" s="23" t="s">
+      <c r="B17" s="18" t="s">
         <v>349</v>
       </c>
-      <c r="C17" s="26" t="s">
+      <c r="C17" s="21" t="s">
         <v>368</v>
       </c>
-      <c r="D17" s="23" t="s">
+      <c r="D17" s="18" t="s">
         <v>369</v>
       </c>
-      <c r="E17" s="23" t="s">
+      <c r="E17" s="18" t="s">
         <v>370</v>
       </c>
-      <c r="F17" s="32" t="s">
-        <v>90</v>
-      </c>
-      <c r="G17" s="26" t="s">
+      <c r="F17" s="27" t="s">
+        <v>90</v>
+      </c>
+      <c r="G17" s="21" t="s">
         <v>97</v>
       </c>
-      <c r="H17" s="26" t="s">
-        <v>86</v>
-      </c>
-      <c r="I17" s="23"/>
+      <c r="H17" s="21" t="s">
+        <v>86</v>
+      </c>
+      <c r="I17" s="18"/>
     </row>
     <row r="18" spans="1:9" ht="51" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="27">
+      <c r="A18" s="22">
         <v>14</v>
       </c>
-      <c r="B18" s="24" t="s">
+      <c r="B18" s="19" t="s">
         <v>371</v>
       </c>
-      <c r="C18" s="27" t="s">
+      <c r="C18" s="22" t="s">
         <v>372</v>
       </c>
-      <c r="D18" s="24" t="s">
+      <c r="D18" s="19" t="s">
         <v>373</v>
       </c>
-      <c r="E18" s="24" t="s">
+      <c r="E18" s="19" t="s">
         <v>374</v>
       </c>
-      <c r="F18" s="36" t="s">
-        <v>90</v>
-      </c>
-      <c r="G18" s="27" t="s">
-        <v>90</v>
-      </c>
-      <c r="H18" s="27" t="s">
-        <v>86</v>
-      </c>
-      <c r="I18" s="24"/>
+      <c r="F18" s="31" t="s">
+        <v>90</v>
+      </c>
+      <c r="G18" s="22" t="s">
+        <v>90</v>
+      </c>
+      <c r="H18" s="22" t="s">
+        <v>86</v>
+      </c>
+      <c r="I18" s="19"/>
     </row>
     <row r="19" spans="1:9" ht="51" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="28">
+      <c r="A19" s="23">
         <v>15</v>
       </c>
-      <c r="B19" s="22" t="s">
+      <c r="B19" s="17" t="s">
         <v>371</v>
       </c>
-      <c r="C19" s="28" t="s">
+      <c r="C19" s="23" t="s">
         <v>375</v>
       </c>
-      <c r="D19" s="22" t="s">
+      <c r="D19" s="17" t="s">
         <v>376</v>
       </c>
-      <c r="E19" s="22" t="s">
+      <c r="E19" s="17" t="s">
         <v>377</v>
       </c>
-      <c r="F19" s="34" t="s">
-        <v>90</v>
-      </c>
-      <c r="G19" s="28" t="s">
+      <c r="F19" s="29" t="s">
+        <v>90</v>
+      </c>
+      <c r="G19" s="23" t="s">
         <v>97</v>
       </c>
-      <c r="H19" s="28" t="s">
-        <v>86</v>
-      </c>
-      <c r="I19" s="22"/>
+      <c r="H19" s="23" t="s">
+        <v>86</v>
+      </c>
+      <c r="I19" s="17"/>
     </row>
     <row r="20" spans="1:9" ht="51" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="25">
+      <c r="A20" s="20">
         <v>16</v>
       </c>
-      <c r="B20" s="7" t="s">
+      <c r="B20" s="12" t="s">
         <v>371</v>
       </c>
-      <c r="C20" s="25" t="s">
+      <c r="C20" s="20" t="s">
         <v>378</v>
       </c>
-      <c r="D20" s="7" t="s">
+      <c r="D20" s="12" t="s">
         <v>379</v>
       </c>
-      <c r="E20" s="7" t="s">
+      <c r="E20" s="12" t="s">
         <v>380</v>
       </c>
-      <c r="F20" s="31" t="s">
-        <v>90</v>
-      </c>
-      <c r="G20" s="25" t="s">
+      <c r="F20" s="26" t="s">
+        <v>90</v>
+      </c>
+      <c r="G20" s="20" t="s">
         <v>97</v>
       </c>
-      <c r="H20" s="25" t="s">
-        <v>86</v>
-      </c>
-      <c r="I20" s="7"/>
+      <c r="H20" s="20" t="s">
+        <v>86</v>
+      </c>
+      <c r="I20" s="12"/>
     </row>
     <row r="21" spans="1:9" ht="51" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="25">
+      <c r="A21" s="20">
         <v>17</v>
       </c>
-      <c r="B21" s="7" t="s">
+      <c r="B21" s="12" t="s">
         <v>371</v>
       </c>
-      <c r="C21" s="25" t="s">
+      <c r="C21" s="20" t="s">
         <v>381</v>
       </c>
-      <c r="D21" s="7" t="s">
+      <c r="D21" s="12" t="s">
         <v>382</v>
       </c>
-      <c r="E21" s="7" t="s">
+      <c r="E21" s="12" t="s">
         <v>383</v>
       </c>
-      <c r="F21" s="31" t="s">
-        <v>90</v>
-      </c>
-      <c r="G21" s="25" t="s">
+      <c r="F21" s="26" t="s">
+        <v>90</v>
+      </c>
+      <c r="G21" s="20" t="s">
         <v>97</v>
       </c>
-      <c r="H21" s="25" t="s">
-        <v>86</v>
-      </c>
-      <c r="I21" s="7"/>
+      <c r="H21" s="20" t="s">
+        <v>86</v>
+      </c>
+      <c r="I21" s="12"/>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">

</xml_diff>

<commit_message>
docs(correcciones): paquete de Esteban completo en correcciones-esteban (44 errores)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Correcciones/Reparto_Correcciones.xlsx
+++ b/Correcciones/Reparto_Correcciones.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/04056fffbf4849c6/Desktop/Estudios/Ingenieria en Sistemas/Ultimo Cuatri/Implantacion/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="48" documentId="8_{8F8D4389-595E-4CF9-BD61-29F667513908}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{479AA629-332A-4350-BE21-47EF3B914DB9}"/>
+  <xr:revisionPtr revIDLastSave="88" documentId="8_{8F8D4389-595E-4CF9-BD61-29F667513908}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E96A4D9B-E9E8-4724-B8A7-BFB43AB40848}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{02318C6D-03B9-4FBB-AC05-EEF1D4A56137}"/>
   </bookViews>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="781" uniqueCount="409">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="801" uniqueCount="429">
   <si>
     <t>Reparto de correcciones — Distribuidora JJ / Licorera La Bodega</t>
   </si>
@@ -1293,6 +1293,66 @@
   </si>
   <si>
     <t>Aviso al chofer al reasignar la ruta (campana web y app). Migración 0221</t>
+  </si>
+  <si>
+    <t>El checkout avisa y no crea el pedido si el stock no alcanza</t>
+  </si>
+  <si>
+    <t>Facturas y estado de cuenta con facturas y pagos en el portal. Migración 0232</t>
+  </si>
+  <si>
+    <t>Estado de cuenta y facturas descargables en PDF real</t>
+  </si>
+  <si>
+    <t>El historial de devoluciones muestra pedido y cliente</t>
+  </si>
+  <si>
+    <t>Reporte de devoluciones por producto, cliente y motivo</t>
+  </si>
+  <si>
+    <t>Pedido a crédito en Venta móvil; bloqueo por deuda vencida (plazo 30 días, pagos FIFO); el cargo es el total facturado con IVA. Migración 0230</t>
+  </si>
+  <si>
+    <t>No se inactiva un cliente con saldo pendiente. Migración 0231</t>
+  </si>
+  <si>
+    <t>El detalle del cliente muestra facturas y saldo (misma consulta que el portal)</t>
+  </si>
+  <si>
+    <t>Contrato de comodato en PDF al asignar. Migración 0244</t>
+  </si>
+  <si>
+    <t>Cliente elegido de la lista y bloqueo por deuda vencida (regla de crédito 0230). Migración 0245</t>
+  </si>
+  <si>
+    <t>Aviso a taller y cobros al devolver un equipo con avería. Migración 0243</t>
+  </si>
+  <si>
+    <t>Regla de 30 días sin compras y alerta de baja rentabilidad. Migración 0242</t>
+  </si>
+  <si>
+    <t>El historial muestra la condición de entrega y de devolución. Migración 0240</t>
+  </si>
+  <si>
+    <t>El reporte muestra ubicación y fecha de entrega. Migración 0241</t>
+  </si>
+  <si>
+    <t>Venta móvil sugiere un artículo complementario</t>
+  </si>
+  <si>
+    <t>Paso a paso de devoluciones, rutas y facturas; rutas de ayuda según el menú actual</t>
+  </si>
+  <si>
+    <t>Cuenta las paradas pendientes de rutas despachadas. Migración 0250</t>
+  </si>
+  <si>
+    <t>Entiende preguntas de ventas y muestra "Información restringida" al Chofer</t>
+  </si>
+  <si>
+    <t>Mensaje "Escribe una pregunta." al enviar vacío</t>
+  </si>
+  <si>
+    <t>Exporta la conversación a Excel (.xlsx)</t>
   </si>
 </sst>
 </file>
@@ -1569,15 +1629,15 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -1682,6 +1742,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2020,17 +2084,17 @@
       </c>
     </row>
     <row r="2" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="39" t="s">
+      <c r="A2" s="38" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="39"/>
-      <c r="C2" s="39"/>
-      <c r="D2" s="39"/>
-      <c r="E2" s="39"/>
-      <c r="F2" s="39"/>
-      <c r="G2" s="39"/>
-      <c r="H2" s="39"/>
-      <c r="I2" s="39"/>
+      <c r="B2" s="38"/>
+      <c r="C2" s="38"/>
+      <c r="D2" s="38"/>
+      <c r="E2" s="38"/>
+      <c r="F2" s="38"/>
+      <c r="G2" s="38"/>
+      <c r="H2" s="38"/>
+      <c r="I2" s="38"/>
     </row>
     <row r="4" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="11" t="s">
@@ -2211,95 +2275,95 @@
       </c>
     </row>
     <row r="12" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="37" t="s">
+      <c r="A12" s="40" t="s">
         <v>29</v>
       </c>
-      <c r="B12" s="37"/>
-      <c r="C12" s="37"/>
-      <c r="D12" s="37"/>
-      <c r="E12" s="37"/>
-      <c r="F12" s="37"/>
-      <c r="G12" s="37"/>
-      <c r="H12" s="37"/>
-      <c r="I12" s="37"/>
+      <c r="B12" s="40"/>
+      <c r="C12" s="40"/>
+      <c r="D12" s="40"/>
+      <c r="E12" s="40"/>
+      <c r="F12" s="40"/>
+      <c r="G12" s="40"/>
+      <c r="H12" s="40"/>
+      <c r="I12" s="40"/>
     </row>
     <row r="13" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="37" t="s">
+      <c r="A13" s="40" t="s">
         <v>30</v>
       </c>
-      <c r="B13" s="37"/>
-      <c r="C13" s="37"/>
-      <c r="D13" s="37"/>
-      <c r="E13" s="37"/>
-      <c r="F13" s="37"/>
-      <c r="G13" s="37"/>
-      <c r="H13" s="37"/>
-      <c r="I13" s="37"/>
+      <c r="B13" s="40"/>
+      <c r="C13" s="40"/>
+      <c r="D13" s="40"/>
+      <c r="E13" s="40"/>
+      <c r="F13" s="40"/>
+      <c r="G13" s="40"/>
+      <c r="H13" s="40"/>
+      <c r="I13" s="40"/>
     </row>
     <row r="14" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="37" t="s">
+      <c r="A14" s="40" t="s">
         <v>31</v>
       </c>
-      <c r="B14" s="37"/>
-      <c r="C14" s="37"/>
-      <c r="D14" s="37"/>
-      <c r="E14" s="37"/>
-      <c r="F14" s="37"/>
-      <c r="G14" s="37"/>
-      <c r="H14" s="37"/>
-      <c r="I14" s="37"/>
+      <c r="B14" s="40"/>
+      <c r="C14" s="40"/>
+      <c r="D14" s="40"/>
+      <c r="E14" s="40"/>
+      <c r="F14" s="40"/>
+      <c r="G14" s="40"/>
+      <c r="H14" s="40"/>
+      <c r="I14" s="40"/>
     </row>
     <row r="15" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="37" t="s">
+      <c r="A15" s="40" t="s">
         <v>32</v>
       </c>
-      <c r="B15" s="37"/>
-      <c r="C15" s="37"/>
-      <c r="D15" s="37"/>
-      <c r="E15" s="37"/>
-      <c r="F15" s="37"/>
-      <c r="G15" s="37"/>
-      <c r="H15" s="37"/>
-      <c r="I15" s="37"/>
+      <c r="B15" s="40"/>
+      <c r="C15" s="40"/>
+      <c r="D15" s="40"/>
+      <c r="E15" s="40"/>
+      <c r="F15" s="40"/>
+      <c r="G15" s="40"/>
+      <c r="H15" s="40"/>
+      <c r="I15" s="40"/>
     </row>
     <row r="16" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="37" t="s">
+      <c r="A16" s="40" t="s">
         <v>33</v>
       </c>
-      <c r="B16" s="37"/>
-      <c r="C16" s="37"/>
-      <c r="D16" s="37"/>
-      <c r="E16" s="37"/>
-      <c r="F16" s="37"/>
-      <c r="G16" s="37"/>
-      <c r="H16" s="37"/>
-      <c r="I16" s="37"/>
+      <c r="B16" s="40"/>
+      <c r="C16" s="40"/>
+      <c r="D16" s="40"/>
+      <c r="E16" s="40"/>
+      <c r="F16" s="40"/>
+      <c r="G16" s="40"/>
+      <c r="H16" s="40"/>
+      <c r="I16" s="40"/>
     </row>
     <row r="17" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="37" t="s">
+      <c r="A17" s="40" t="s">
         <v>34</v>
       </c>
-      <c r="B17" s="37"/>
-      <c r="C17" s="37"/>
-      <c r="D17" s="37"/>
-      <c r="E17" s="37"/>
-      <c r="F17" s="37"/>
-      <c r="G17" s="37"/>
-      <c r="H17" s="37"/>
-      <c r="I17" s="37"/>
+      <c r="B17" s="40"/>
+      <c r="C17" s="40"/>
+      <c r="D17" s="40"/>
+      <c r="E17" s="40"/>
+      <c r="F17" s="40"/>
+      <c r="G17" s="40"/>
+      <c r="H17" s="40"/>
+      <c r="I17" s="40"/>
     </row>
     <row r="18" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="37" t="s">
+      <c r="A18" s="40" t="s">
         <v>35</v>
       </c>
-      <c r="B18" s="37"/>
-      <c r="C18" s="37"/>
-      <c r="D18" s="37"/>
-      <c r="E18" s="37"/>
-      <c r="F18" s="37"/>
-      <c r="G18" s="37"/>
-      <c r="H18" s="37"/>
-      <c r="I18" s="37"/>
+      <c r="B18" s="40"/>
+      <c r="C18" s="40"/>
+      <c r="D18" s="40"/>
+      <c r="E18" s="40"/>
+      <c r="F18" s="40"/>
+      <c r="G18" s="40"/>
+      <c r="H18" s="40"/>
+      <c r="I18" s="40"/>
     </row>
     <row r="20" spans="1:9" ht="17.25" x14ac:dyDescent="0.3">
       <c r="A20" s="10" t="s">
@@ -2330,15 +2394,15 @@
       <c r="B22" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="C22" s="40" t="s">
+      <c r="C22" s="39" t="s">
         <v>42</v>
       </c>
-      <c r="D22" s="40"/>
-      <c r="E22" s="40"/>
-      <c r="F22" s="40"/>
-      <c r="G22" s="40"/>
-      <c r="H22" s="40"/>
-      <c r="I22" s="40"/>
+      <c r="D22" s="39"/>
+      <c r="E22" s="39"/>
+      <c r="F22" s="39"/>
+      <c r="G22" s="39"/>
+      <c r="H22" s="39"/>
+      <c r="I22" s="39"/>
     </row>
     <row r="23" spans="1:9" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
@@ -2347,15 +2411,15 @@
       <c r="B23" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="C23" s="40" t="s">
+      <c r="C23" s="39" t="s">
         <v>44</v>
       </c>
-      <c r="D23" s="40"/>
-      <c r="E23" s="40"/>
-      <c r="F23" s="40"/>
-      <c r="G23" s="40"/>
-      <c r="H23" s="40"/>
-      <c r="I23" s="40"/>
+      <c r="D23" s="39"/>
+      <c r="E23" s="39"/>
+      <c r="F23" s="39"/>
+      <c r="G23" s="39"/>
+      <c r="H23" s="39"/>
+      <c r="I23" s="39"/>
     </row>
     <row r="24" spans="1:9" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
@@ -2364,15 +2428,15 @@
       <c r="B24" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="C24" s="40" t="s">
+      <c r="C24" s="39" t="s">
         <v>47</v>
       </c>
-      <c r="D24" s="40"/>
-      <c r="E24" s="40"/>
-      <c r="F24" s="40"/>
-      <c r="G24" s="40"/>
-      <c r="H24" s="40"/>
-      <c r="I24" s="40"/>
+      <c r="D24" s="39"/>
+      <c r="E24" s="39"/>
+      <c r="F24" s="39"/>
+      <c r="G24" s="39"/>
+      <c r="H24" s="39"/>
+      <c r="I24" s="39"/>
     </row>
     <row r="25" spans="1:9" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
@@ -2381,15 +2445,15 @@
       <c r="B25" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="C25" s="40" t="s">
+      <c r="C25" s="39" t="s">
         <v>49</v>
       </c>
-      <c r="D25" s="40"/>
-      <c r="E25" s="40"/>
-      <c r="F25" s="40"/>
-      <c r="G25" s="40"/>
-      <c r="H25" s="40"/>
-      <c r="I25" s="40"/>
+      <c r="D25" s="39"/>
+      <c r="E25" s="39"/>
+      <c r="F25" s="39"/>
+      <c r="G25" s="39"/>
+      <c r="H25" s="39"/>
+      <c r="I25" s="39"/>
     </row>
     <row r="26" spans="1:9" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="5" t="s">
@@ -2398,15 +2462,15 @@
       <c r="B26" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="C26" s="40" t="s">
+      <c r="C26" s="39" t="s">
         <v>52</v>
       </c>
-      <c r="D26" s="40"/>
-      <c r="E26" s="40"/>
-      <c r="F26" s="40"/>
-      <c r="G26" s="40"/>
-      <c r="H26" s="40"/>
-      <c r="I26" s="40"/>
+      <c r="D26" s="39"/>
+      <c r="E26" s="39"/>
+      <c r="F26" s="39"/>
+      <c r="G26" s="39"/>
+      <c r="H26" s="39"/>
+      <c r="I26" s="39"/>
     </row>
     <row r="28" spans="1:9" ht="17.25" x14ac:dyDescent="0.3">
       <c r="A28" s="10" t="s">
@@ -2417,124 +2481,130 @@
       <c r="A29" s="13" t="s">
         <v>54</v>
       </c>
-      <c r="B29" s="38" t="s">
+      <c r="B29" s="37" t="s">
         <v>55</v>
       </c>
-      <c r="C29" s="38"/>
-      <c r="D29" s="38"/>
-      <c r="E29" s="38"/>
-      <c r="F29" s="38"/>
-      <c r="G29" s="38"/>
-      <c r="H29" s="38"/>
-      <c r="I29" s="38"/>
+      <c r="C29" s="37"/>
+      <c r="D29" s="37"/>
+      <c r="E29" s="37"/>
+      <c r="F29" s="37"/>
+      <c r="G29" s="37"/>
+      <c r="H29" s="37"/>
+      <c r="I29" s="37"/>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" s="14" t="s">
         <v>56</v>
       </c>
-      <c r="B30" s="38" t="s">
+      <c r="B30" s="37" t="s">
         <v>57</v>
       </c>
-      <c r="C30" s="38"/>
-      <c r="D30" s="38"/>
-      <c r="E30" s="38"/>
-      <c r="F30" s="38"/>
-      <c r="G30" s="38"/>
-      <c r="H30" s="38"/>
-      <c r="I30" s="38"/>
+      <c r="C30" s="37"/>
+      <c r="D30" s="37"/>
+      <c r="E30" s="37"/>
+      <c r="F30" s="37"/>
+      <c r="G30" s="37"/>
+      <c r="H30" s="37"/>
+      <c r="I30" s="37"/>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" s="15" t="s">
         <v>58</v>
       </c>
-      <c r="B31" s="38" t="s">
+      <c r="B31" s="37" t="s">
         <v>59</v>
       </c>
-      <c r="C31" s="38"/>
-      <c r="D31" s="38"/>
-      <c r="E31" s="38"/>
-      <c r="F31" s="38"/>
-      <c r="G31" s="38"/>
-      <c r="H31" s="38"/>
-      <c r="I31" s="38"/>
+      <c r="C31" s="37"/>
+      <c r="D31" s="37"/>
+      <c r="E31" s="37"/>
+      <c r="F31" s="37"/>
+      <c r="G31" s="37"/>
+      <c r="H31" s="37"/>
+      <c r="I31" s="37"/>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="B32" s="38" t="s">
+      <c r="B32" s="37" t="s">
         <v>61</v>
       </c>
-      <c r="C32" s="38"/>
-      <c r="D32" s="38"/>
-      <c r="E32" s="38"/>
-      <c r="F32" s="38"/>
-      <c r="G32" s="38"/>
-      <c r="H32" s="38"/>
-      <c r="I32" s="38"/>
+      <c r="C32" s="37"/>
+      <c r="D32" s="37"/>
+      <c r="E32" s="37"/>
+      <c r="F32" s="37"/>
+      <c r="G32" s="37"/>
+      <c r="H32" s="37"/>
+      <c r="I32" s="37"/>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="B33" s="38" t="s">
+      <c r="B33" s="37" t="s">
         <v>63</v>
       </c>
-      <c r="C33" s="38"/>
-      <c r="D33" s="38"/>
-      <c r="E33" s="38"/>
-      <c r="F33" s="38"/>
-      <c r="G33" s="38"/>
-      <c r="H33" s="38"/>
-      <c r="I33" s="38"/>
+      <c r="C33" s="37"/>
+      <c r="D33" s="37"/>
+      <c r="E33" s="37"/>
+      <c r="F33" s="37"/>
+      <c r="G33" s="37"/>
+      <c r="H33" s="37"/>
+      <c r="I33" s="37"/>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="B34" s="38" t="s">
+      <c r="B34" s="37" t="s">
         <v>65</v>
       </c>
-      <c r="C34" s="38"/>
-      <c r="D34" s="38"/>
-      <c r="E34" s="38"/>
-      <c r="F34" s="38"/>
-      <c r="G34" s="38"/>
-      <c r="H34" s="38"/>
-      <c r="I34" s="38"/>
+      <c r="C34" s="37"/>
+      <c r="D34" s="37"/>
+      <c r="E34" s="37"/>
+      <c r="F34" s="37"/>
+      <c r="G34" s="37"/>
+      <c r="H34" s="37"/>
+      <c r="I34" s="37"/>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B35" s="38" t="s">
+      <c r="B35" s="37" t="s">
         <v>66</v>
       </c>
-      <c r="C35" s="38"/>
-      <c r="D35" s="38"/>
-      <c r="E35" s="38"/>
-      <c r="F35" s="38"/>
-      <c r="G35" s="38"/>
-      <c r="H35" s="38"/>
-      <c r="I35" s="38"/>
+      <c r="C35" s="37"/>
+      <c r="D35" s="37"/>
+      <c r="E35" s="37"/>
+      <c r="F35" s="37"/>
+      <c r="G35" s="37"/>
+      <c r="H35" s="37"/>
+      <c r="I35" s="37"/>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="B36" s="38" t="s">
+      <c r="B36" s="37" t="s">
         <v>68</v>
       </c>
-      <c r="C36" s="38"/>
-      <c r="D36" s="38"/>
-      <c r="E36" s="38"/>
-      <c r="F36" s="38"/>
-      <c r="G36" s="38"/>
-      <c r="H36" s="38"/>
-      <c r="I36" s="38"/>
+      <c r="C36" s="37"/>
+      <c r="D36" s="37"/>
+      <c r="E36" s="37"/>
+      <c r="F36" s="37"/>
+      <c r="G36" s="37"/>
+      <c r="H36" s="37"/>
+      <c r="I36" s="37"/>
     </row>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="A17:I17"/>
+    <mergeCell ref="A12:I12"/>
+    <mergeCell ref="A13:I13"/>
+    <mergeCell ref="A14:I14"/>
+    <mergeCell ref="A15:I15"/>
+    <mergeCell ref="A16:I16"/>
     <mergeCell ref="B34:I34"/>
     <mergeCell ref="B35:I35"/>
     <mergeCell ref="B36:I36"/>
@@ -2551,12 +2621,6 @@
     <mergeCell ref="C23:I23"/>
     <mergeCell ref="C24:I24"/>
     <mergeCell ref="C25:I25"/>
-    <mergeCell ref="A17:I17"/>
-    <mergeCell ref="A12:I12"/>
-    <mergeCell ref="A13:I13"/>
-    <mergeCell ref="A14:I14"/>
-    <mergeCell ref="A15:I15"/>
-    <mergeCell ref="A16:I16"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup fitToHeight="0" orientation="landscape" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
@@ -2587,17 +2651,17 @@
       </c>
     </row>
     <row r="2" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="39" t="s">
+      <c r="A2" s="38" t="s">
         <v>70</v>
       </c>
-      <c r="B2" s="39"/>
-      <c r="C2" s="39"/>
-      <c r="D2" s="39"/>
-      <c r="E2" s="39"/>
-      <c r="F2" s="39"/>
-      <c r="G2" s="39"/>
-      <c r="H2" s="39"/>
-      <c r="I2" s="39"/>
+      <c r="B2" s="38"/>
+      <c r="C2" s="38"/>
+      <c r="D2" s="38"/>
+      <c r="E2" s="38"/>
+      <c r="F2" s="38"/>
+      <c r="G2" s="38"/>
+      <c r="H2" s="38"/>
+      <c r="I2" s="38"/>
     </row>
     <row r="4" spans="1:9" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="11" t="s">
@@ -2883,9 +2947,11 @@
         <v>85</v>
       </c>
       <c r="H13" s="22" t="s">
-        <v>86</v>
-      </c>
-      <c r="I13" s="19"/>
+        <v>384</v>
+      </c>
+      <c r="I13" s="19" t="s">
+        <v>409</v>
+      </c>
     </row>
     <row r="14" spans="1:9" ht="81" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="23">
@@ -2939,9 +3005,11 @@
         <v>90</v>
       </c>
       <c r="H15" s="20" t="s">
-        <v>86</v>
-      </c>
-      <c r="I15" s="12"/>
+        <v>384</v>
+      </c>
+      <c r="I15" s="12" t="s">
+        <v>410</v>
+      </c>
     </row>
     <row r="16" spans="1:9" ht="51" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="21">
@@ -2966,9 +3034,11 @@
         <v>90</v>
       </c>
       <c r="H16" s="21" t="s">
-        <v>86</v>
-      </c>
-      <c r="I16" s="18"/>
+        <v>384</v>
+      </c>
+      <c r="I16" s="18" t="s">
+        <v>411</v>
+      </c>
     </row>
     <row r="17" spans="1:9" ht="66" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="22">
@@ -2993,9 +3063,11 @@
         <v>97</v>
       </c>
       <c r="H17" s="22" t="s">
-        <v>86</v>
-      </c>
-      <c r="I17" s="19"/>
+        <v>384</v>
+      </c>
+      <c r="I17" s="19" t="s">
+        <v>412</v>
+      </c>
     </row>
     <row r="18" spans="1:9" ht="51" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="24">
@@ -3020,9 +3092,11 @@
         <v>90</v>
       </c>
       <c r="H18" s="24" t="s">
-        <v>86</v>
-      </c>
-      <c r="I18" s="16"/>
+        <v>384</v>
+      </c>
+      <c r="I18" s="16" t="s">
+        <v>413</v>
+      </c>
     </row>
     <row r="19" spans="1:9" ht="51" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="22">
@@ -3047,9 +3121,11 @@
         <v>85</v>
       </c>
       <c r="H19" s="22" t="s">
-        <v>86</v>
-      </c>
-      <c r="I19" s="19"/>
+        <v>384</v>
+      </c>
+      <c r="I19" s="19" t="s">
+        <v>414</v>
+      </c>
     </row>
     <row r="20" spans="1:9" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="23">
@@ -3074,9 +3150,11 @@
         <v>90</v>
       </c>
       <c r="H20" s="23" t="s">
-        <v>86</v>
-      </c>
-      <c r="I20" s="17"/>
+        <v>384</v>
+      </c>
+      <c r="I20" s="17" t="s">
+        <v>415</v>
+      </c>
     </row>
     <row r="21" spans="1:9" ht="36" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="21">
@@ -3101,9 +3179,11 @@
         <v>90</v>
       </c>
       <c r="H21" s="21" t="s">
-        <v>86</v>
-      </c>
-      <c r="I21" s="18"/>
+        <v>384</v>
+      </c>
+      <c r="I21" s="18" t="s">
+        <v>416</v>
+      </c>
     </row>
     <row r="22" spans="1:9" ht="51" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="22">
@@ -3128,9 +3208,11 @@
         <v>85</v>
       </c>
       <c r="H22" s="22" t="s">
-        <v>86</v>
-      </c>
-      <c r="I22" s="19"/>
+        <v>384</v>
+      </c>
+      <c r="I22" s="19" t="s">
+        <v>417</v>
+      </c>
     </row>
     <row r="23" spans="1:9" ht="51" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="23">
@@ -3155,9 +3237,11 @@
         <v>90</v>
       </c>
       <c r="H23" s="23" t="s">
-        <v>86</v>
-      </c>
-      <c r="I23" s="17"/>
+        <v>384</v>
+      </c>
+      <c r="I23" s="17" t="s">
+        <v>418</v>
+      </c>
     </row>
     <row r="24" spans="1:9" ht="51" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="20">
@@ -3182,9 +3266,11 @@
         <v>90</v>
       </c>
       <c r="H24" s="20" t="s">
-        <v>86</v>
-      </c>
-      <c r="I24" s="12"/>
+        <v>384</v>
+      </c>
+      <c r="I24" s="12" t="s">
+        <v>419</v>
+      </c>
     </row>
     <row r="25" spans="1:9" ht="51" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="20">
@@ -3209,9 +3295,11 @@
         <v>90</v>
       </c>
       <c r="H25" s="20" t="s">
-        <v>86</v>
-      </c>
-      <c r="I25" s="12"/>
+        <v>384</v>
+      </c>
+      <c r="I25" s="12" t="s">
+        <v>420</v>
+      </c>
     </row>
     <row r="26" spans="1:9" ht="51" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="20">
@@ -3236,9 +3324,11 @@
         <v>97</v>
       </c>
       <c r="H26" s="20" t="s">
-        <v>86</v>
-      </c>
-      <c r="I26" s="12"/>
+        <v>384</v>
+      </c>
+      <c r="I26" s="12" t="s">
+        <v>421</v>
+      </c>
     </row>
     <row r="27" spans="1:9" ht="51" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="21">
@@ -3263,9 +3353,11 @@
         <v>97</v>
       </c>
       <c r="H27" s="21" t="s">
-        <v>86</v>
-      </c>
-      <c r="I27" s="18"/>
+        <v>384</v>
+      </c>
+      <c r="I27" s="18" t="s">
+        <v>422</v>
+      </c>
     </row>
     <row r="28" spans="1:9" ht="66" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="22">
@@ -3406,9 +3498,11 @@
         <v>90</v>
       </c>
       <c r="H32" s="22" t="s">
-        <v>86</v>
-      </c>
-      <c r="I32" s="19"/>
+        <v>384</v>
+      </c>
+      <c r="I32" s="19" t="s">
+        <v>423</v>
+      </c>
     </row>
     <row r="33" spans="1:9" ht="81" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="23">
@@ -3433,9 +3527,11 @@
         <v>90</v>
       </c>
       <c r="H33" s="23" t="s">
-        <v>86</v>
-      </c>
-      <c r="I33" s="17"/>
+        <v>384</v>
+      </c>
+      <c r="I33" s="17" t="s">
+        <v>424</v>
+      </c>
     </row>
     <row r="34" spans="1:9" ht="51" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="20">
@@ -3460,9 +3556,11 @@
         <v>90</v>
       </c>
       <c r="H34" s="20" t="s">
-        <v>86</v>
-      </c>
-      <c r="I34" s="12"/>
+        <v>384</v>
+      </c>
+      <c r="I34" s="12" t="s">
+        <v>425</v>
+      </c>
     </row>
     <row r="35" spans="1:9" ht="66" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="20">
@@ -3487,9 +3585,11 @@
         <v>90</v>
       </c>
       <c r="H35" s="20" t="s">
-        <v>86</v>
-      </c>
-      <c r="I35" s="12"/>
+        <v>384</v>
+      </c>
+      <c r="I35" s="12" t="s">
+        <v>426</v>
+      </c>
     </row>
     <row r="36" spans="1:9" ht="51" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="20">
@@ -3514,9 +3614,11 @@
         <v>97</v>
       </c>
       <c r="H36" s="20" t="s">
-        <v>86</v>
-      </c>
-      <c r="I36" s="12"/>
+        <v>384</v>
+      </c>
+      <c r="I36" s="12" t="s">
+        <v>427</v>
+      </c>
     </row>
     <row r="37" spans="1:9" ht="51" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="21">
@@ -3541,9 +3643,11 @@
         <v>97</v>
       </c>
       <c r="H37" s="21" t="s">
-        <v>86</v>
-      </c>
-      <c r="I37" s="18"/>
+        <v>384</v>
+      </c>
+      <c r="I37" s="18" t="s">
+        <v>428</v>
+      </c>
     </row>
     <row r="38" spans="1:9" ht="51" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="22">
@@ -3870,7 +3974,7 @@
       </c>
       <c r="B50" s="2" t="str">
         <f>COUNTIF(H5:H48,"Corregido")&amp;" de 44 corregidos"</f>
-        <v>24 de 44 corregidos</v>
+        <v>44 de 44 corregidos</v>
       </c>
     </row>
   </sheetData>
@@ -3930,17 +4034,17 @@
       </c>
     </row>
     <row r="2" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="39" t="s">
+      <c r="A2" s="38" t="s">
         <v>229</v>
       </c>
-      <c r="B2" s="39"/>
-      <c r="C2" s="39"/>
-      <c r="D2" s="39"/>
-      <c r="E2" s="39"/>
-      <c r="F2" s="39"/>
-      <c r="G2" s="39"/>
-      <c r="H2" s="39"/>
-      <c r="I2" s="39"/>
+      <c r="B2" s="38"/>
+      <c r="C2" s="38"/>
+      <c r="D2" s="38"/>
+      <c r="E2" s="38"/>
+      <c r="F2" s="38"/>
+      <c r="G2" s="38"/>
+      <c r="H2" s="38"/>
+      <c r="I2" s="38"/>
     </row>
     <row r="4" spans="1:9" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="11" t="s">
@@ -4469,17 +4573,17 @@
       </c>
     </row>
     <row r="2" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="39" t="s">
+      <c r="A2" s="38" t="s">
         <v>281</v>
       </c>
-      <c r="B2" s="39"/>
-      <c r="C2" s="39"/>
-      <c r="D2" s="39"/>
-      <c r="E2" s="39"/>
-      <c r="F2" s="39"/>
-      <c r="G2" s="39"/>
-      <c r="H2" s="39"/>
-      <c r="I2" s="39"/>
+      <c r="B2" s="38"/>
+      <c r="C2" s="38"/>
+      <c r="D2" s="38"/>
+      <c r="E2" s="38"/>
+      <c r="F2" s="38"/>
+      <c r="G2" s="38"/>
+      <c r="H2" s="38"/>
+      <c r="I2" s="38"/>
     </row>
     <row r="4" spans="1:9" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="11" t="s">
@@ -4954,17 +5058,17 @@
       </c>
     </row>
     <row r="2" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="39" t="s">
+      <c r="A2" s="38" t="s">
         <v>329</v>
       </c>
-      <c r="B2" s="39"/>
-      <c r="C2" s="39"/>
-      <c r="D2" s="39"/>
-      <c r="E2" s="39"/>
-      <c r="F2" s="39"/>
-      <c r="G2" s="39"/>
-      <c r="H2" s="39"/>
-      <c r="I2" s="39"/>
+      <c r="B2" s="38"/>
+      <c r="C2" s="38"/>
+      <c r="D2" s="38"/>
+      <c r="E2" s="38"/>
+      <c r="F2" s="38"/>
+      <c r="G2" s="38"/>
+      <c r="H2" s="38"/>
+      <c r="I2" s="38"/>
     </row>
     <row r="4" spans="1:9" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="11" t="s">

</xml_diff>